<commit_message>
atualiza volumes loa com ppo - 15092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
+++ b/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
@@ -63035,7 +63035,7 @@
         </is>
       </c>
       <c r="U907" t="n">
-        <v>224028722</v>
+        <v>224028723</v>
       </c>
       <c r="V907" t="n">
         <v>2027</v>
@@ -63104,7 +63104,7 @@
         </is>
       </c>
       <c r="U908" t="n">
-        <v>52709660</v>
+        <v>52709658</v>
       </c>
       <c r="V908" t="n">
         <v>2027</v>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 18092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
+++ b/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
@@ -29639,7 +29639,7 @@
         </is>
       </c>
       <c r="U423" t="n">
-        <v>136984940</v>
+        <v>36984940</v>
       </c>
       <c r="V423" t="n">
         <v>2027</v>
@@ -29708,7 +29708,7 @@
         </is>
       </c>
       <c r="U424" t="n">
-        <v>210621931</v>
+        <v>67470413</v>
       </c>
       <c r="V424" t="n">
         <v>2027</v>
@@ -29777,7 +29777,7 @@
         </is>
       </c>
       <c r="U425" t="n">
-        <v>304901962</v>
+        <v>404901962</v>
       </c>
       <c r="V425" t="n">
         <v>2027</v>
@@ -29846,7 +29846,7 @@
         </is>
       </c>
       <c r="U426" t="n">
-        <v>468803654</v>
+        <v>611955172</v>
       </c>
       <c r="V426" t="n">
         <v>2027</v>
@@ -31571,7 +31571,7 @@
         </is>
       </c>
       <c r="U451" t="n">
-        <v>428116013</v>
+        <v>489300262</v>
       </c>
       <c r="V451" t="n">
         <v>2027</v>
@@ -31709,7 +31709,7 @@
         </is>
       </c>
       <c r="U453" t="n">
-        <v>952903383</v>
+        <v>891719134</v>
       </c>
       <c r="V453" t="n">
         <v>2027</v>
@@ -59723,7 +59723,7 @@
         </is>
       </c>
       <c r="U859" t="n">
-        <v>278049881</v>
+        <v>274549881</v>
       </c>
       <c r="V859" t="n">
         <v>2027</v>
@@ -59792,7 +59792,7 @@
         </is>
       </c>
       <c r="U860" t="n">
-        <v>15642849</v>
+        <v>20642849</v>
       </c>
       <c r="V860" t="n">
         <v>2027</v>
@@ -59999,7 +59999,7 @@
         </is>
       </c>
       <c r="U863" t="n">
-        <v>-15642849</v>
+        <v>-20642849</v>
       </c>
       <c r="V863" t="n">
         <v>2027</v>
@@ -77525,7 +77525,7 @@
         </is>
       </c>
       <c r="U1117" t="n">
-        <v>89164234</v>
+        <v>117664234</v>
       </c>
       <c r="V1117" t="n">
         <v>2027</v>
@@ -81251,7 +81251,7 @@
         </is>
       </c>
       <c r="U1171" t="n">
-        <v>364800957</v>
+        <v>390963136</v>
       </c>
       <c r="V1171" t="n">
         <v>2027</v>
@@ -81282,22 +81282,22 @@
         </is>
       </c>
       <c r="D1172" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1172" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H1172" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I1172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J1172" t="n">
         <v>2</v>
       </c>
       <c r="K1172" t="n">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="L1172" t="n">
         <v>0</v>
@@ -81306,21 +81306,21 @@
         <v>1</v>
       </c>
       <c r="N1172" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="O1172" t="n">
         <v>0</v>
       </c>
       <c r="P1172" t="n">
-        <v>7922990199000</v>
+        <v>9112510102000</v>
       </c>
       <c r="Q1172" t="inlineStr">
         <is>
-          <t>REC. INTRA. - OUTRAS RESTITUIÇÕES - PRINC. - DEMAIS</t>
+          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1172" t="n">
-        <v>1000</v>
+        <v>-6730265620</v>
       </c>
       <c r="V1172" t="n">
         <v>2027</v>
@@ -81332,7 +81332,7 @@
       </c>
       <c r="X1172" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81351,7 +81351,7 @@
         </is>
       </c>
       <c r="D1173" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1173" t="n">
         <v>9</v>
@@ -81375,21 +81375,21 @@
         <v>1</v>
       </c>
       <c r="N1173" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1173" t="n">
         <v>0</v>
       </c>
       <c r="P1173" t="n">
-        <v>9112510102000</v>
+        <v>9112510103000</v>
       </c>
       <c r="Q1173" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1173" t="n">
-        <v>-6730265620</v>
+        <v>-1346053124</v>
       </c>
       <c r="V1173" t="n">
         <v>2027</v>
@@ -81401,7 +81401,7 @@
       </c>
       <c r="X1173" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81420,7 +81420,7 @@
         </is>
       </c>
       <c r="D1174" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1174" t="n">
         <v>9</v>
@@ -81441,24 +81441,24 @@
         <v>0</v>
       </c>
       <c r="M1174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1174" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1174" t="n">
         <v>0</v>
       </c>
       <c r="P1174" t="n">
-        <v>9112510103000</v>
+        <v>9112510202000</v>
       </c>
       <c r="Q1174" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1174" t="n">
-        <v>-1346053124</v>
+        <v>-440382545</v>
       </c>
       <c r="V1174" t="n">
         <v>2027</v>
@@ -81470,7 +81470,7 @@
       </c>
       <c r="X1174" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81489,7 +81489,7 @@
         </is>
       </c>
       <c r="D1175" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1175" t="n">
         <v>9</v>
@@ -81513,21 +81513,21 @@
         <v>2</v>
       </c>
       <c r="N1175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1175" t="n">
         <v>0</v>
       </c>
       <c r="P1175" t="n">
-        <v>9112510202000</v>
+        <v>9112510203000</v>
       </c>
       <c r="Q1175" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1175" t="n">
-        <v>-440382545</v>
+        <v>-88076509</v>
       </c>
       <c r="V1175" t="n">
         <v>2027</v>
@@ -81539,7 +81539,7 @@
       </c>
       <c r="X1175" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81558,7 +81558,7 @@
         </is>
       </c>
       <c r="D1176" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1176" t="n">
         <v>9</v>
@@ -81579,24 +81579,24 @@
         <v>0</v>
       </c>
       <c r="M1176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1176" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1176" t="n">
         <v>0</v>
       </c>
       <c r="P1176" t="n">
-        <v>9112510203000</v>
+        <v>9112510302000</v>
       </c>
       <c r="Q1176" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1176" t="n">
-        <v>-88076509</v>
+        <v>-176418275</v>
       </c>
       <c r="V1176" t="n">
         <v>2027</v>
@@ -81608,7 +81608,7 @@
       </c>
       <c r="X1176" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81627,7 +81627,7 @@
         </is>
       </c>
       <c r="D1177" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1177" t="n">
         <v>9</v>
@@ -81651,21 +81651,21 @@
         <v>3</v>
       </c>
       <c r="N1177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1177" t="n">
         <v>0</v>
       </c>
       <c r="P1177" t="n">
-        <v>9112510302000</v>
+        <v>9112510303000</v>
       </c>
       <c r="Q1177" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1177" t="n">
-        <v>-176418275</v>
+        <v>-35283655</v>
       </c>
       <c r="V1177" t="n">
         <v>2027</v>
@@ -81677,7 +81677,7 @@
       </c>
       <c r="X1177" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81711,30 +81711,30 @@
         <v>2</v>
       </c>
       <c r="K1178" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L1178" t="n">
         <v>0</v>
       </c>
       <c r="M1178" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1178" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1178" t="n">
         <v>0</v>
       </c>
       <c r="P1178" t="n">
-        <v>9112510303000</v>
+        <v>9112520102000</v>
       </c>
       <c r="Q1178" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1178" t="n">
-        <v>-35283655</v>
+        <v>-469496703</v>
       </c>
       <c r="V1178" t="n">
         <v>2027</v>
@@ -81746,7 +81746,7 @@
       </c>
       <c r="X1178" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81786,7 +81786,7 @@
         <v>0</v>
       </c>
       <c r="M1179" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1179" t="n">
         <v>2</v>
@@ -81795,15 +81795,15 @@
         <v>0</v>
       </c>
       <c r="P1179" t="n">
-        <v>9112520102000</v>
+        <v>9112520202000</v>
       </c>
       <c r="Q1179" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1179" t="n">
-        <v>-469496703</v>
+        <v>-39568452</v>
       </c>
       <c r="V1179" t="n">
         <v>2027</v>
@@ -81815,7 +81815,7 @@
       </c>
       <c r="X1179" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81855,7 +81855,7 @@
         <v>0</v>
       </c>
       <c r="M1180" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1180" t="n">
         <v>2</v>
@@ -81864,15 +81864,15 @@
         <v>0</v>
       </c>
       <c r="P1180" t="n">
-        <v>9112520202000</v>
+        <v>9112520302000</v>
       </c>
       <c r="Q1180" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1180" t="n">
-        <v>-39568452</v>
+        <v>-6352385</v>
       </c>
       <c r="V1180" t="n">
         <v>2027</v>
@@ -81884,7 +81884,7 @@
       </c>
       <c r="X1180" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81903,7 +81903,7 @@
         </is>
       </c>
       <c r="D1181" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1181" t="n">
         <v>9</v>
@@ -81915,33 +81915,33 @@
         <v>1</v>
       </c>
       <c r="J1181" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K1181" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L1181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1181" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1181" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O1181" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1181" t="n">
-        <v>9112520302000</v>
+        <v>9114501101002</v>
       </c>
       <c r="Q1181" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1181" t="n">
-        <v>-6352385</v>
+        <v>-328488</v>
       </c>
       <c r="V1181" t="n">
         <v>2027</v>
@@ -81953,7 +81953,7 @@
       </c>
       <c r="X1181" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -81972,7 +81972,7 @@
         </is>
       </c>
       <c r="D1182" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1182" t="n">
         <v>9</v>
@@ -81996,21 +81996,21 @@
         <v>1</v>
       </c>
       <c r="N1182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1182" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1182" t="n">
-        <v>9114501101002</v>
+        <v>9114501102000</v>
       </c>
       <c r="Q1182" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1182" t="n">
-        <v>-328488</v>
+        <v>-23077484102</v>
       </c>
       <c r="V1182" t="n">
         <v>2027</v>
@@ -82022,7 +82022,7 @@
       </c>
       <c r="X1182" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -82041,7 +82041,7 @@
         </is>
       </c>
       <c r="D1183" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1183" t="n">
         <v>9</v>
@@ -82065,21 +82065,21 @@
         <v>1</v>
       </c>
       <c r="N1183" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1183" t="n">
         <v>0</v>
       </c>
       <c r="P1183" t="n">
-        <v>9114501102000</v>
+        <v>9114501103000</v>
       </c>
       <c r="Q1183" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1183" t="n">
-        <v>-23077484102</v>
+        <v>-13846490461</v>
       </c>
       <c r="V1183" t="n">
         <v>2027</v>
@@ -82091,7 +82091,7 @@
       </c>
       <c r="X1183" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82110,7 +82110,7 @@
         </is>
       </c>
       <c r="D1184" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1184" t="n">
         <v>9</v>
@@ -82131,24 +82131,24 @@
         <v>1</v>
       </c>
       <c r="M1184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1184" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O1184" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1184" t="n">
-        <v>9114501103000</v>
+        <v>9114501201002</v>
       </c>
       <c r="Q1184" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1184" t="n">
-        <v>-13846490461</v>
+        <v>-638942</v>
       </c>
       <c r="V1184" t="n">
         <v>2027</v>
@@ -82160,7 +82160,7 @@
       </c>
       <c r="X1184" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -82179,7 +82179,7 @@
         </is>
       </c>
       <c r="D1185" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1185" t="n">
         <v>9</v>
@@ -82203,21 +82203,21 @@
         <v>2</v>
       </c>
       <c r="N1185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1185" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1185" t="n">
-        <v>9114501201002</v>
+        <v>9114501202000</v>
       </c>
       <c r="Q1185" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1185" t="n">
-        <v>-638942</v>
+        <v>-255087472</v>
       </c>
       <c r="V1185" t="n">
         <v>2027</v>
@@ -82229,7 +82229,7 @@
       </c>
       <c r="X1185" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -82248,7 +82248,7 @@
         </is>
       </c>
       <c r="D1186" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1186" t="n">
         <v>9</v>
@@ -82272,21 +82272,21 @@
         <v>2</v>
       </c>
       <c r="N1186" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1186" t="n">
         <v>0</v>
       </c>
       <c r="P1186" t="n">
-        <v>9114501202000</v>
+        <v>9114501203000</v>
       </c>
       <c r="Q1186" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1186" t="n">
-        <v>-255087472</v>
+        <v>-153052483</v>
       </c>
       <c r="V1186" t="n">
         <v>2027</v>
@@ -82298,7 +82298,7 @@
       </c>
       <c r="X1186" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82317,7 +82317,7 @@
         </is>
       </c>
       <c r="D1187" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1187" t="n">
         <v>9</v>
@@ -82338,24 +82338,24 @@
         <v>1</v>
       </c>
       <c r="M1187" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1187" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O1187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1187" t="n">
-        <v>9114501203000</v>
+        <v>9114501301002</v>
       </c>
       <c r="Q1187" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1187" t="n">
-        <v>-153052483</v>
+        <v>-7869701</v>
       </c>
       <c r="V1187" t="n">
         <v>2027</v>
@@ -82367,7 +82367,7 @@
       </c>
       <c r="X1187" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -82386,7 +82386,7 @@
         </is>
       </c>
       <c r="D1188" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1188" t="n">
         <v>9</v>
@@ -82410,21 +82410,21 @@
         <v>3</v>
       </c>
       <c r="N1188" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1188" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1188" t="n">
-        <v>9114501301002</v>
+        <v>9114501302000</v>
       </c>
       <c r="Q1188" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1188" t="n">
-        <v>-7869701</v>
+        <v>-201596219</v>
       </c>
       <c r="V1188" t="n">
         <v>2027</v>
@@ -82436,7 +82436,7 @@
       </c>
       <c r="X1188" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -82455,7 +82455,7 @@
         </is>
       </c>
       <c r="D1189" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1189" t="n">
         <v>9</v>
@@ -82479,21 +82479,21 @@
         <v>3</v>
       </c>
       <c r="N1189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1189" t="n">
         <v>0</v>
       </c>
       <c r="P1189" t="n">
-        <v>9114501302000</v>
+        <v>9114501303000</v>
       </c>
       <c r="Q1189" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1189" t="n">
-        <v>-201596219</v>
+        <v>-120957732</v>
       </c>
       <c r="V1189" t="n">
         <v>2027</v>
@@ -82505,7 +82505,7 @@
       </c>
       <c r="X1189" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82542,27 +82542,27 @@
         <v>50</v>
       </c>
       <c r="L1190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M1190" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1190" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1190" t="n">
         <v>0</v>
       </c>
       <c r="P1190" t="n">
-        <v>9114501303000</v>
+        <v>9114502102000</v>
       </c>
       <c r="Q1190" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ADICIONAL ICMS - FEM - PRINC. - COTA PARTE DO FUNDEB</t>
         </is>
       </c>
       <c r="U1190" t="n">
-        <v>-120957732</v>
+        <v>-224000000</v>
       </c>
       <c r="V1190" t="n">
         <v>2027</v>
@@ -82574,7 +82574,7 @@
       </c>
       <c r="X1190" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -82593,7 +82593,7 @@
         </is>
       </c>
       <c r="D1191" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1191" t="n">
         <v>9</v>
@@ -82605,13 +82605,13 @@
         <v>1</v>
       </c>
       <c r="J1191" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K1191" t="n">
         <v>50</v>
       </c>
       <c r="L1191" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M1191" t="n">
         <v>1</v>
@@ -82623,15 +82623,15 @@
         <v>0</v>
       </c>
       <c r="P1191" t="n">
-        <v>9114502102000</v>
+        <v>9116500102000</v>
       </c>
       <c r="Q1191" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ADICIONAL ICMS - FEM - PRINC. - COTA PARTE DO FUNDEB</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1191" t="n">
-        <v>-224000000</v>
+        <v>-64413502</v>
       </c>
       <c r="V1191" t="n">
         <v>2027</v>
@@ -82643,7 +82643,7 @@
       </c>
       <c r="X1191" t="inlineStr">
         <is>
-          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Inclui IBS - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -82662,7 +82662,7 @@
         </is>
       </c>
       <c r="D1192" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1192" t="n">
         <v>9</v>
@@ -82686,21 +82686,21 @@
         <v>1</v>
       </c>
       <c r="N1192" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1192" t="n">
         <v>0</v>
       </c>
       <c r="P1192" t="n">
-        <v>9116500102000</v>
+        <v>9116500103000</v>
       </c>
       <c r="Q1192" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1192" t="n">
-        <v>-64413502</v>
+        <v>-38648102</v>
       </c>
       <c r="V1192" t="n">
         <v>2027</v>
@@ -82731,7 +82731,7 @@
         </is>
       </c>
       <c r="D1193" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1193" t="n">
         <v>9</v>
@@ -82755,21 +82755,21 @@
         <v>1</v>
       </c>
       <c r="N1193" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O1193" t="n">
         <v>0</v>
       </c>
       <c r="P1193" t="n">
-        <v>9116500103000</v>
+        <v>9116500104000</v>
       </c>
       <c r="Q1193" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O COMITÊ GESTOR DO IBS</t>
         </is>
       </c>
       <c r="U1193" t="n">
-        <v>-38648102</v>
+        <v>-96620253</v>
       </c>
       <c r="V1193" t="n">
         <v>2027</v>
@@ -82800,19 +82800,19 @@
         </is>
       </c>
       <c r="D1194" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1194" t="n">
         <v>9</v>
       </c>
       <c r="H1194" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I1194" t="n">
         <v>1</v>
       </c>
       <c r="J1194" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K1194" t="n">
         <v>50</v>
@@ -82824,21 +82824,21 @@
         <v>1</v>
       </c>
       <c r="N1194" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O1194" t="n">
         <v>0</v>
       </c>
       <c r="P1194" t="n">
-        <v>9116500104000</v>
+        <v>9711500102000</v>
       </c>
       <c r="Q1194" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O COMITÊ GESTOR DO IBS</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE FPE - PRINC. - FUNDEB</t>
         </is>
       </c>
       <c r="U1194" t="n">
-        <v>-96620253</v>
+        <v>-2099559983</v>
       </c>
       <c r="V1194" t="n">
         <v>2027</v>
@@ -82850,7 +82850,7 @@
       </c>
       <c r="X1194" t="inlineStr">
         <is>
-          <t>Inclui IBS - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Receita de Dedução Receita - Cota-Parte FPE - Princ. - FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82869,7 +82869,7 @@
         </is>
       </c>
       <c r="D1195" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1195" t="n">
         <v>9</v>
@@ -82884,7 +82884,7 @@
         <v>1</v>
       </c>
       <c r="K1195" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="L1195" t="n">
         <v>0</v>
@@ -82899,15 +82899,15 @@
         <v>0</v>
       </c>
       <c r="P1195" t="n">
-        <v>9711500102000</v>
+        <v>9711530102000</v>
       </c>
       <c r="Q1195" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE FPE - PRINC. - FUNDEB</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1195" t="n">
-        <v>-2099559983</v>
+        <v>-330174995</v>
       </c>
       <c r="V1195" t="n">
         <v>2027</v>
@@ -82919,7 +82919,7 @@
       </c>
       <c r="X1195" t="inlineStr">
         <is>
-          <t>Receita de Dedução Receita - Cota-Parte FPE - Princ. - FUNDEB</t>
+          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - Municípios.</t>
         </is>
       </c>
     </row>
@@ -82938,7 +82938,7 @@
         </is>
       </c>
       <c r="D1196" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1196" t="n">
         <v>9</v>
@@ -82962,21 +82962,21 @@
         <v>1</v>
       </c>
       <c r="N1196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1196" t="n">
         <v>0</v>
       </c>
       <c r="P1196" t="n">
-        <v>9711530102000</v>
+        <v>9711530103000</v>
       </c>
       <c r="Q1196" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - FUNDEB</t>
         </is>
       </c>
       <c r="U1196" t="n">
-        <v>-330174995</v>
+        <v>-198104997</v>
       </c>
       <c r="V1196" t="n">
         <v>2027</v>
@@ -82988,7 +82988,7 @@
       </c>
       <c r="X1196" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - Municípios.</t>
+          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - FUNDEB</t>
         </is>
       </c>
     </row>
@@ -83007,7 +83007,7 @@
         </is>
       </c>
       <c r="D1197" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G1197" t="n">
         <v>9</v>
@@ -83022,7 +83022,7 @@
         <v>1</v>
       </c>
       <c r="K1197" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L1197" t="n">
         <v>0</v>
@@ -83031,21 +83031,21 @@
         <v>1</v>
       </c>
       <c r="N1197" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1197" t="n">
         <v>0</v>
       </c>
       <c r="P1197" t="n">
-        <v>9711530103000</v>
+        <v>9711540102000</v>
       </c>
       <c r="Q1197" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - FUNDEB</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE CIDE - PRINC. - MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1197" t="n">
-        <v>-198104997</v>
+        <v>-29360522</v>
       </c>
       <c r="V1197" t="n">
         <v>2027</v>
@@ -83057,7 +83057,7 @@
       </c>
       <c r="X1197" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - FUNDEB</t>
+          <t>Receita de Dedução Receita - Cota-Parte CIDE - Princ. - Municípios</t>
         </is>
       </c>
     </row>
@@ -83076,13 +83076,13 @@
         </is>
       </c>
       <c r="D1198" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="G1198" t="n">
         <v>9</v>
       </c>
       <c r="H1198" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I1198" t="n">
         <v>1</v>
@@ -83091,7 +83091,7 @@
         <v>1</v>
       </c>
       <c r="K1198" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="L1198" t="n">
         <v>0</v>
@@ -83100,21 +83100,21 @@
         <v>1</v>
       </c>
       <c r="N1198" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1198" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P1198" t="n">
-        <v>9711540102000</v>
+        <v>9911010103004</v>
       </c>
       <c r="Q1198" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE CIDE - PRINC. - MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
         </is>
       </c>
       <c r="U1198" t="n">
-        <v>-29360522</v>
+        <v>-11702813</v>
       </c>
       <c r="V1198" t="n">
         <v>2027</v>
@@ -83125,75 +83125,6 @@
         </is>
       </c>
       <c r="X1198" t="inlineStr">
-        <is>
-          <t>Receita de Dedução Receita - Cota-Parte CIDE - Princ. - Municípios</t>
-        </is>
-      </c>
-    </row>
-    <row r="1199">
-      <c r="A1199" t="n">
-        <v>9901</v>
-      </c>
-      <c r="B1199" t="inlineStr">
-        <is>
-          <t>RECEITA GERAL DO ESTADO</t>
-        </is>
-      </c>
-      <c r="C1199" t="inlineStr">
-        <is>
-          <t>RGE</t>
-        </is>
-      </c>
-      <c r="D1199" t="n">
-        <v>82</v>
-      </c>
-      <c r="G1199" t="n">
-        <v>9</v>
-      </c>
-      <c r="H1199" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1199" t="n">
-        <v>1</v>
-      </c>
-      <c r="J1199" t="n">
-        <v>1</v>
-      </c>
-      <c r="K1199" t="n">
-        <v>1</v>
-      </c>
-      <c r="L1199" t="n">
-        <v>0</v>
-      </c>
-      <c r="M1199" t="n">
-        <v>1</v>
-      </c>
-      <c r="N1199" t="n">
-        <v>3</v>
-      </c>
-      <c r="O1199" t="n">
-        <v>4</v>
-      </c>
-      <c r="P1199" t="n">
-        <v>9911010103004</v>
-      </c>
-      <c r="Q1199" t="inlineStr">
-        <is>
-          <t>DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
-        </is>
-      </c>
-      <c r="U1199" t="n">
-        <v>-11702813</v>
-      </c>
-      <c r="V1199" t="n">
-        <v>2027</v>
-      </c>
-      <c r="W1199" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X1199" t="inlineStr">
         <is>
           <t>RECeita de DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
         </is>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 21092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
+++ b/bancos/SISOR/BASE_ORCAM_RECEITA_FISCAL.xlsx
@@ -9491,7 +9491,7 @@
         </is>
       </c>
       <c r="U131" t="n">
-        <v>186957216</v>
+        <v>191718584</v>
       </c>
       <c r="V131" t="n">
         <v>2027</v>
@@ -10005,7 +10005,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G139" t="n">
         <v>1</v>
@@ -10017,10 +10017,10 @@
         <v>1</v>
       </c>
       <c r="J139" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K139" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L139" t="n">
         <v>0</v>
@@ -10029,21 +10029,21 @@
         <v>1</v>
       </c>
       <c r="N139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O139" t="n">
         <v>0</v>
       </c>
       <c r="P139" t="n">
-        <v>1715530101000</v>
+        <v>1717510102000</v>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>TRANSF. FUNDEB MATRÍCULAS ETI - PRINC.</t>
+          <t>EDUCAÇÃO - INSTITUTO NACIONAL DE ESTUDOS E PESQUISAS EDUCACIONAIS ANÍSIO TEIXEIRA - INEP</t>
         </is>
       </c>
       <c r="U139" t="n">
-        <v>4761368</v>
+        <v>294865</v>
       </c>
       <c r="V139" t="n">
         <v>2027</v>
@@ -10055,7 +10055,7 @@
       </c>
       <c r="X139" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)  </t>
+          <t>VALOR ESTIMADO COM BASE NOS INSTRUMENTOS JURÍDICOS VIGENTES, NAS RESPECTIVAS PREVISÕES DE INGRESSO DE RECURSOS E, QUANDO APLICÁVEL, EM PROPOSTAS DE NOVOS INSTRUMENTOS EM ANÁLISE OU EM FASE DE FORMALIZAÇÃO JUNTO AOS CONCEDENTES.</t>
         </is>
       </c>
     </row>
@@ -10074,7 +10074,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G140" t="n">
         <v>1</v>
@@ -10083,13 +10083,13 @@
         <v>7</v>
       </c>
       <c r="I140" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J140" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K140" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L140" t="n">
         <v>0</v>
@@ -10098,21 +10098,21 @@
         <v>1</v>
       </c>
       <c r="N140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O140" t="n">
         <v>0</v>
       </c>
       <c r="P140" t="n">
-        <v>1717510102000</v>
+        <v>1751500101000</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>EDUCAÇÃO - INSTITUTO NACIONAL DE ESTUDOS E PESQUISAS EDUCACIONAIS ANÍSIO TEIXEIRA - INEP</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA FPM</t>
         </is>
       </c>
       <c r="U140" t="n">
-        <v>294865</v>
+        <v>2676120990</v>
       </c>
       <c r="V140" t="n">
         <v>2027</v>
@@ -10124,7 +10124,7 @@
       </c>
       <c r="X140" t="inlineStr">
         <is>
-          <t>VALOR ESTIMADO COM BASE NOS INSTRUMENTOS JURÍDICOS VIGENTES, NAS RESPECTIVAS PREVISÕES DE INGRESSO DE RECURSOS E, QUANDO APLICÁVEL, EM PROPOSTAS DE NOVOS INSTRUMENTOS EM ANÁLISE OU EM FASE DE FORMALIZAÇÃO JUNTO AOS CONCEDENTES.</t>
+          <t xml:space="preserve"> Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)  </t>
         </is>
       </c>
     </row>
@@ -10167,21 +10167,21 @@
         <v>1</v>
       </c>
       <c r="N141" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P141" t="n">
-        <v>1751500101000</v>
+        <v>1751500103001</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA FPM</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - PRINC.</t>
         </is>
       </c>
       <c r="U141" t="n">
-        <v>2676120990</v>
+        <v>8031822881</v>
       </c>
       <c r="V141" t="n">
         <v>2027</v>
@@ -10239,18 +10239,18 @@
         <v>3</v>
       </c>
       <c r="O142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P142" t="n">
-        <v>1751500103001</v>
+        <v>1751500103002</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - MULTAS E JUROS</t>
         </is>
       </c>
       <c r="U142" t="n">
-        <v>8031822881</v>
+        <v>88779929</v>
       </c>
       <c r="V142" t="n">
         <v>2027</v>
@@ -10262,7 +10262,7 @@
       </c>
       <c r="X142" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)  </t>
+          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
         </is>
       </c>
     </row>
@@ -10308,18 +10308,18 @@
         <v>3</v>
       </c>
       <c r="O143" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P143" t="n">
-        <v>1751500103002</v>
+        <v>1751500103003</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - MULTAS E JUROS</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - DA</t>
         </is>
       </c>
       <c r="U143" t="n">
-        <v>88779929</v>
+        <v>70162983</v>
       </c>
       <c r="V143" t="n">
         <v>2027</v>
@@ -10374,21 +10374,21 @@
         <v>1</v>
       </c>
       <c r="N144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O144" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P144" t="n">
-        <v>1751500103003</v>
+        <v>1751500104001</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ICMS - DA</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPI - PRINC.</t>
         </is>
       </c>
       <c r="U144" t="n">
-        <v>70162983</v>
+        <v>114913180</v>
       </c>
       <c r="V144" t="n">
         <v>2027</v>
@@ -10443,21 +10443,21 @@
         <v>1</v>
       </c>
       <c r="N145" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O145" t="n">
         <v>1</v>
       </c>
       <c r="P145" t="n">
-        <v>1751500104001</v>
+        <v>1751500105001</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPI - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA FPE - PRINC.</t>
         </is>
       </c>
       <c r="U145" t="n">
-        <v>114913180</v>
+        <v>913406214</v>
       </c>
       <c r="V145" t="n">
         <v>2027</v>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="X145" t="inlineStr">
         <is>
-          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
+          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%).</t>
         </is>
       </c>
     </row>
@@ -10512,21 +10512,21 @@
         <v>1</v>
       </c>
       <c r="N146" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O146" t="n">
         <v>1</v>
       </c>
       <c r="P146" t="n">
-        <v>1751500105001</v>
+        <v>1751500106001</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA FPE - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITR - PRINC.</t>
         </is>
       </c>
       <c r="U146" t="n">
-        <v>913406214</v>
+        <v>10270643</v>
       </c>
       <c r="V146" t="n">
         <v>2027</v>
@@ -10581,21 +10581,21 @@
         <v>1</v>
       </c>
       <c r="N147" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O147" t="n">
         <v>1</v>
       </c>
       <c r="P147" t="n">
-        <v>1751500106001</v>
+        <v>1751500107001</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITR - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - PRINC.</t>
         </is>
       </c>
       <c r="U147" t="n">
-        <v>10270643</v>
+        <v>1171191391</v>
       </c>
       <c r="V147" t="n">
         <v>2027</v>
@@ -10653,18 +10653,18 @@
         <v>7</v>
       </c>
       <c r="O148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P148" t="n">
-        <v>1751500107001</v>
+        <v>1751500107002</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - MULTAS E JUROS</t>
         </is>
       </c>
       <c r="U148" t="n">
-        <v>1171191391</v>
+        <v>76634753</v>
       </c>
       <c r="V148" t="n">
         <v>2027</v>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="X148" t="inlineStr">
         <is>
-          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%).</t>
+          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
         </is>
       </c>
     </row>
@@ -10722,18 +10722,18 @@
         <v>7</v>
       </c>
       <c r="O149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P149" t="n">
-        <v>1751500107002</v>
+        <v>1751500107003</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - MULTAS E JUROS</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - DA</t>
         </is>
       </c>
       <c r="U149" t="n">
-        <v>76634753</v>
+        <v>30700061</v>
       </c>
       <c r="V149" t="n">
         <v>2027</v>
@@ -10788,21 +10788,21 @@
         <v>1</v>
       </c>
       <c r="N150" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O150" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P150" t="n">
-        <v>1751500107003</v>
+        <v>1751500108001</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IPVA - DA</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - PRINC.</t>
         </is>
       </c>
       <c r="U150" t="n">
-        <v>30700061</v>
+        <v>204252896</v>
       </c>
       <c r="V150" t="n">
         <v>2027</v>
@@ -10814,7 +10814,7 @@
       </c>
       <c r="X150" t="inlineStr">
         <is>
-          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
+          <t xml:space="preserve">Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%). </t>
         </is>
       </c>
     </row>
@@ -10860,18 +10860,18 @@
         <v>8</v>
       </c>
       <c r="O151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P151" t="n">
-        <v>1751500108001</v>
+        <v>1751500108002</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - MULTAS E JUROS</t>
         </is>
       </c>
       <c r="U151" t="n">
-        <v>204252896</v>
+        <v>17214116</v>
       </c>
       <c r="V151" t="n">
         <v>2027</v>
@@ -10883,7 +10883,7 @@
       </c>
       <c r="X151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%). </t>
+          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
         </is>
       </c>
     </row>
@@ -10929,18 +10929,18 @@
         <v>8</v>
       </c>
       <c r="O152" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P152" t="n">
-        <v>1751500108002</v>
+        <v>1751500108003</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - MULTAS E JUROS</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - DA</t>
         </is>
       </c>
       <c r="U152" t="n">
-        <v>17214116</v>
+        <v>2763583</v>
       </c>
       <c r="V152" t="n">
         <v>2027</v>
@@ -10995,21 +10995,21 @@
         <v>1</v>
       </c>
       <c r="N153" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P153" t="n">
-        <v>1751500108003</v>
+        <v>1751500109001</v>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ITCD - DA</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ADICIONAL ICMS - FEM - PRINC.</t>
         </is>
       </c>
       <c r="U153" t="n">
-        <v>2763583</v>
+        <v>97450415</v>
       </c>
       <c r="V153" t="n">
         <v>2027</v>
@@ -11021,7 +11021,7 @@
       </c>
       <c r="X153" t="inlineStr">
         <is>
-          <t>Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%)</t>
+          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -11067,18 +11067,18 @@
         <v>9</v>
       </c>
       <c r="O154" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P154" t="n">
-        <v>1751500109001</v>
+        <v>1751500109005</v>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ADICIONAL ICMS - FEM - PRINC.</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ADICIONAL ICMS - FEM - EXERCÍCIOS ANTERIORES</t>
         </is>
       </c>
       <c r="U154" t="n">
-        <v>97450415</v>
+        <v>162484816</v>
       </c>
       <c r="V154" t="n">
         <v>2027</v>
@@ -11090,7 +11090,7 @@
       </c>
       <c r="X154" t="inlineStr">
         <is>
-          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t xml:space="preserve">Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%). </t>
         </is>
       </c>
     </row>
@@ -11133,21 +11133,21 @@
         <v>1</v>
       </c>
       <c r="N155" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O155" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P155" t="n">
-        <v>1751500109005</v>
+        <v>1751500112000</v>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA ADICIONAL ICMS - FEM - EXERCÍCIOS ANTERIORES</t>
+          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IBS</t>
         </is>
       </c>
       <c r="U155" t="n">
-        <v>162484816</v>
+        <v>22429769</v>
       </c>
       <c r="V155" t="n">
         <v>2027</v>
@@ -11159,7 +11159,7 @@
       </c>
       <c r="X155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor estimado para o exercício de 2027 com base no montante arrecadado em 2025 versus o IPCA projetado pelo Banco Central do Brasil para o ano de 2026. (Relatório Focus - 4,7%). </t>
+          <t>Reforma tributária nacional que institui o IBS como imposto estadual.</t>
         </is>
       </c>
     </row>
@@ -16598,7 +16598,7 @@
         </is>
       </c>
       <c r="U234" t="n">
-        <v>8591486</v>
+        <v>683000</v>
       </c>
       <c r="V234" t="n">
         <v>2027</v>
@@ -18599,7 +18599,7 @@
         </is>
       </c>
       <c r="U263" t="n">
-        <v>228137430</v>
+        <v>273050387</v>
       </c>
       <c r="V263" t="n">
         <v>2027</v>
@@ -20393,7 +20393,7 @@
         </is>
       </c>
       <c r="U289" t="n">
-        <v>32920516</v>
+        <v>32456131</v>
       </c>
       <c r="V289" t="n">
         <v>2027</v>
@@ -35849,7 +35849,7 @@
         </is>
       </c>
       <c r="U513" t="n">
-        <v>673587524</v>
+        <v>660792564</v>
       </c>
       <c r="V513" t="n">
         <v>2027</v>
@@ -37298,7 +37298,7 @@
         </is>
       </c>
       <c r="U534" t="n">
-        <v>2567858752</v>
+        <v>2659579770</v>
       </c>
       <c r="V534" t="n">
         <v>2027</v>
@@ -40265,7 +40265,7 @@
         </is>
       </c>
       <c r="U577" t="n">
-        <v>1038</v>
+        <v>65002000</v>
       </c>
       <c r="V577" t="n">
         <v>2027</v>
@@ -41990,7 +41990,7 @@
         </is>
       </c>
       <c r="U602" t="n">
-        <v>429513701</v>
+        <v>431909937</v>
       </c>
       <c r="V602" t="n">
         <v>2027</v>
@@ -54203,7 +54203,7 @@
         </is>
       </c>
       <c r="U779" t="n">
-        <v>6927209</v>
+        <v>0</v>
       </c>
       <c r="V779" t="n">
         <v>2027</v>
@@ -62345,7 +62345,7 @@
         </is>
       </c>
       <c r="U897" t="n">
-        <v>1038</v>
+        <v>986428</v>
       </c>
       <c r="V897" t="n">
         <v>2027</v>
@@ -74489,7 +74489,7 @@
         </is>
       </c>
       <c r="U1073" t="n">
-        <v>1312101799</v>
+        <v>1312849799</v>
       </c>
       <c r="V1073" t="n">
         <v>2027</v>
@@ -77211,22 +77211,22 @@
         </is>
       </c>
       <c r="D1113" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G1113" t="n">
         <v>1</v>
       </c>
       <c r="H1113" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I1113" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J1113" t="n">
         <v>1</v>
       </c>
       <c r="K1113" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="L1113" t="n">
         <v>0</v>
@@ -77235,21 +77235,21 @@
         <v>1</v>
       </c>
       <c r="N1113" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="O1113" t="n">
         <v>0</v>
       </c>
       <c r="P1113" t="n">
-        <v>1751500112000</v>
+        <v>1911010101000</v>
       </c>
       <c r="Q1113" t="inlineStr">
         <is>
-          <t>TRANSF. RECURSOS FUNDEB - PRINC. - PARCELA IBS</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISLAÇÃO SANITÁRIA</t>
         </is>
       </c>
       <c r="U1113" t="n">
-        <v>22429769</v>
+        <v>229002</v>
       </c>
       <c r="V1113" t="n">
         <v>2027</v>
@@ -77261,7 +77261,7 @@
       </c>
       <c r="X1113" t="inlineStr">
         <is>
-          <t>Inclui IBS - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -77280,7 +77280,7 @@
         </is>
       </c>
       <c r="D1114" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G1114" t="n">
         <v>1</v>
@@ -77304,21 +77304,21 @@
         <v>1</v>
       </c>
       <c r="N1114" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O1114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P1114" t="n">
-        <v>1911010101000</v>
+        <v>1911010103001</v>
       </c>
       <c r="Q1114" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISLAÇÃO SANITÁRIA</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO ESTADO</t>
         </is>
       </c>
       <c r="U1114" t="n">
-        <v>229002</v>
+        <v>66706034</v>
       </c>
       <c r="V1114" t="n">
         <v>2027</v>
@@ -77330,7 +77330,7 @@
       </c>
       <c r="X1114" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Receita de desvinculação - 30% (trinta por cento) da receita desvinculada.</t>
         </is>
       </c>
     </row>
@@ -77349,7 +77349,7 @@
         </is>
       </c>
       <c r="D1115" t="n">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="G1115" t="n">
         <v>1</v>
@@ -77387,7 +77387,7 @@
         </is>
       </c>
       <c r="U1115" t="n">
-        <v>66706034</v>
+        <v>155647413</v>
       </c>
       <c r="V1115" t="n">
         <v>2027</v>
@@ -77399,7 +77399,7 @@
       </c>
       <c r="X1115" t="inlineStr">
         <is>
-          <t>Receita de desvinculação - 30% (trinta por cento) da receita desvinculada.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -77418,7 +77418,7 @@
         </is>
       </c>
       <c r="D1116" t="n">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="G1116" t="n">
         <v>1</v>
@@ -77445,18 +77445,18 @@
         <v>3</v>
       </c>
       <c r="O1116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P1116" t="n">
-        <v>1911010103001</v>
+        <v>1911010103002</v>
       </c>
       <c r="Q1116" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO ESTADO</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO DEPARTAMENTO DE EDIFICAÇÕES E ESTRADAS DE RODAGEM DO ESTADO DE MINAS GERAIS - DERMG</t>
         </is>
       </c>
       <c r="U1116" t="n">
-        <v>155647413</v>
+        <v>117664234</v>
       </c>
       <c r="V1116" t="n">
         <v>2027</v>
@@ -77468,7 +77468,7 @@
       </c>
       <c r="X1116" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
         </is>
       </c>
     </row>
@@ -77487,7 +77487,7 @@
         </is>
       </c>
       <c r="D1117" t="n">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="G1117" t="n">
         <v>1</v>
@@ -77514,18 +77514,18 @@
         <v>3</v>
       </c>
       <c r="O1117" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P1117" t="n">
-        <v>1911010103002</v>
+        <v>1911010103004</v>
       </c>
       <c r="Q1117" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO DEPARTAMENTO DE EDIFICAÇÕES E ESTRADAS DE RODAGEM DO ESTADO DE MINAS GERAIS - DERMG</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
         </is>
       </c>
       <c r="U1117" t="n">
-        <v>117664234</v>
+        <v>11702813</v>
       </c>
       <c r="V1117" t="n">
         <v>2027</v>
@@ -77537,7 +77537,7 @@
       </c>
       <c r="X1117" t="inlineStr">
         <is>
-          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -77556,7 +77556,7 @@
         </is>
       </c>
       <c r="D1118" t="n">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="G1118" t="n">
         <v>1</v>
@@ -77580,21 +77580,21 @@
         <v>1</v>
       </c>
       <c r="N1118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O1118" t="n">
-        <v>4</v>
+        <v>999</v>
       </c>
       <c r="P1118" t="n">
-        <v>1911010103004</v>
+        <v>1911010104999</v>
       </c>
       <c r="Q1118" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
         </is>
       </c>
       <c r="U1118" t="n">
-        <v>11702813</v>
+        <v>50098846</v>
       </c>
       <c r="V1118" t="n">
         <v>2027</v>
@@ -77606,7 +77606,7 @@
       </c>
       <c r="X1118" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Foram projetados tendo por base os valores históricos observados em exercícios recentes (janeiro de 2014 a fevereiro de 2026) e foram utilizados modelos ARIMA e de Alisamento Exponencial.</t>
         </is>
       </c>
     </row>
@@ -77625,7 +77625,7 @@
         </is>
       </c>
       <c r="D1119" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G1119" t="n">
         <v>1</v>
@@ -77649,21 +77649,21 @@
         <v>1</v>
       </c>
       <c r="N1119" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="O1119" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="P1119" t="n">
-        <v>1911010104999</v>
+        <v>1911010112000</v>
       </c>
       <c r="Q1119" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - INFRAÇÃO À LEGISLAÇÃO DE ABASTECIMENTO DE ÁGUA E ESGOTAMENTO SANITÁRIO</t>
         </is>
       </c>
       <c r="U1119" t="n">
-        <v>50098846</v>
+        <v>108665</v>
       </c>
       <c r="V1119" t="n">
         <v>2027</v>
@@ -77675,7 +77675,7 @@
       </c>
       <c r="X1119" t="inlineStr">
         <is>
-          <t>Foram projetados tendo por base os valores históricos observados em exercícios recentes (janeiro de 2014 a fevereiro de 2026) e foram utilizados modelos ARIMA e de Alisamento Exponencial.</t>
+          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
         </is>
       </c>
     </row>
@@ -77694,7 +77694,7 @@
         </is>
       </c>
       <c r="D1120" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G1120" t="n">
         <v>1</v>
@@ -77715,24 +77715,24 @@
         <v>0</v>
       </c>
       <c r="M1120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1120" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="O1120" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="P1120" t="n">
-        <v>1911010112000</v>
+        <v>1911010204999</v>
       </c>
       <c r="Q1120" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - PRINC. - INFRAÇÃO À LEGISLAÇÃO DE ABASTECIMENTO DE ÁGUA E ESGOTAMENTO SANITÁRIO</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - MJM - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
         </is>
       </c>
       <c r="U1120" t="n">
-        <v>108665</v>
+        <v>18238</v>
       </c>
       <c r="V1120" t="n">
         <v>2027</v>
@@ -77744,7 +77744,7 @@
       </c>
       <c r="X1120" t="inlineStr">
         <is>
-          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -77784,7 +77784,7 @@
         <v>0</v>
       </c>
       <c r="M1121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1121" t="n">
         <v>4</v>
@@ -77793,15 +77793,15 @@
         <v>999</v>
       </c>
       <c r="P1121" t="n">
-        <v>1911010204999</v>
+        <v>1911010304999</v>
       </c>
       <c r="Q1121" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - MJM - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - DA - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
         </is>
       </c>
       <c r="U1121" t="n">
-        <v>18238</v>
+        <v>47046653</v>
       </c>
       <c r="V1121" t="n">
         <v>2027</v>
@@ -77853,7 +77853,7 @@
         <v>0</v>
       </c>
       <c r="M1122" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N1122" t="n">
         <v>4</v>
@@ -77862,15 +77862,15 @@
         <v>999</v>
       </c>
       <c r="P1122" t="n">
-        <v>1911010304999</v>
+        <v>1911010404999</v>
       </c>
       <c r="Q1122" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - DA - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
+          <t>MULTAS LEGISL. ESPECÍFICA - DA-MJM - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
         </is>
       </c>
       <c r="U1122" t="n">
-        <v>47046653</v>
+        <v>22142</v>
       </c>
       <c r="V1122" t="n">
         <v>2027</v>
@@ -77916,30 +77916,30 @@
         <v>1</v>
       </c>
       <c r="K1123" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L1123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1123" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N1123" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O1123" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="P1123" t="n">
-        <v>1911010404999</v>
+        <v>1911061101000</v>
       </c>
       <c r="Q1123" t="inlineStr">
         <is>
-          <t>MULTAS LEGISL. ESPECÍFICA - DA-MJM - MULTA ISOLADA OBRIG. ACESSÓRIA - OUTROS</t>
+          <t>MULTAS ADM. DANOS AMBIENTAIS - PRINC.</t>
         </is>
       </c>
       <c r="U1123" t="n">
-        <v>22142</v>
+        <v>136931530</v>
       </c>
       <c r="V1123" t="n">
         <v>2027</v>
@@ -77951,7 +77951,7 @@
       </c>
       <c r="X1123" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Corresponde à Receita Prevista Atualizada de 2026, majorada pelo fator de crescimento esperado do PIB em 2026, 1,6% na estimativa do BACEN.</t>
         </is>
       </c>
     </row>
@@ -77970,7 +77970,7 @@
         </is>
       </c>
       <c r="D1124" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G1124" t="n">
         <v>1</v>
@@ -77985,30 +77985,30 @@
         <v>1</v>
       </c>
       <c r="K1124" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L1124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M1124" t="n">
         <v>1</v>
       </c>
       <c r="N1124" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="O1124" t="n">
         <v>0</v>
       </c>
       <c r="P1124" t="n">
-        <v>1911061101000</v>
+        <v>1911090199000</v>
       </c>
       <c r="Q1124" t="inlineStr">
         <is>
-          <t>MULTAS ADM. DANOS AMBIENTAIS - PRINC.</t>
+          <t>MULTAS JUROS PREVISTOS CONTRATOS - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1124" t="n">
-        <v>136931530</v>
+        <v>1000</v>
       </c>
       <c r="V1124" t="n">
         <v>2027</v>
@@ -78020,7 +78020,7 @@
       </c>
       <c r="X1124" t="inlineStr">
         <is>
-          <t>Corresponde à Receita Prevista Atualizada de 2026, majorada pelo fator de crescimento esperado do PIB em 2026, 1,6% na estimativa do BACEN.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -78039,7 +78039,7 @@
         </is>
       </c>
       <c r="D1125" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G1125" t="n">
         <v>1</v>
@@ -78077,7 +78077,7 @@
         </is>
       </c>
       <c r="U1125" t="n">
-        <v>1000</v>
+        <v>523455</v>
       </c>
       <c r="V1125" t="n">
         <v>2027</v>
@@ -78089,7 +78089,7 @@
       </c>
       <c r="X1125" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -78123,30 +78123,30 @@
         <v>1</v>
       </c>
       <c r="K1126" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L1126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M1126" t="n">
         <v>1</v>
       </c>
       <c r="N1126" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1126" t="n">
         <v>0</v>
       </c>
       <c r="P1126" t="n">
-        <v>1911090199000</v>
+        <v>1911132101000</v>
       </c>
       <c r="Q1126" t="inlineStr">
         <is>
-          <t>MULTAS JUROS PREVISTOS CONTRATOS - PRINC. - DEMAIS</t>
+          <t>MULTAS LEGISLAÇÃO ANTICORRUPÇÃO ACORDOS LENIÊNCIA - PRINC.</t>
         </is>
       </c>
       <c r="U1126" t="n">
-        <v>523455</v>
+        <v>1000</v>
       </c>
       <c r="V1126" t="n">
         <v>2027</v>
@@ -78158,7 +78158,7 @@
       </c>
       <c r="X1126" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -78177,7 +78177,7 @@
         </is>
       </c>
       <c r="D1127" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G1127" t="n">
         <v>1</v>
@@ -78186,16 +78186,16 @@
         <v>9</v>
       </c>
       <c r="I1127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J1127" t="n">
         <v>1</v>
       </c>
       <c r="K1127" t="n">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="L1127" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M1127" t="n">
         <v>1</v>
@@ -78207,15 +78207,15 @@
         <v>0</v>
       </c>
       <c r="P1127" t="n">
-        <v>1911132101000</v>
+        <v>1921990101000</v>
       </c>
       <c r="Q1127" t="inlineStr">
         <is>
-          <t>MULTAS LEGISLAÇÃO ANTICORRUPÇÃO ACORDOS LENIÊNCIA - PRINC.</t>
+          <t>OUTRAS INDENIZAÇÕES - PRINC. - IMPACTOS E DANOS AMBIENTAIS</t>
         </is>
       </c>
       <c r="U1127" t="n">
-        <v>1000</v>
+        <v>7371429</v>
       </c>
       <c r="V1127" t="n">
         <v>2027</v>
@@ -78227,7 +78227,7 @@
       </c>
       <c r="X1127" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
         </is>
       </c>
     </row>
@@ -78246,7 +78246,7 @@
         </is>
       </c>
       <c r="D1128" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G1128" t="n">
         <v>1</v>
@@ -78270,21 +78270,21 @@
         <v>1</v>
       </c>
       <c r="N1128" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="O1128" t="n">
         <v>0</v>
       </c>
       <c r="P1128" t="n">
-        <v>1921990101000</v>
+        <v>1921990199000</v>
       </c>
       <c r="Q1128" t="inlineStr">
         <is>
-          <t>OUTRAS INDENIZAÇÕES - PRINC. - IMPACTOS E DANOS AMBIENTAIS</t>
+          <t>OUTRAS INDENIZAÇÕES - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1128" t="n">
-        <v>7371429</v>
+        <v>2513608</v>
       </c>
       <c r="V1128" t="n">
         <v>2027</v>
@@ -78296,7 +78296,7 @@
       </c>
       <c r="X1128" t="inlineStr">
         <is>
-          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -78315,7 +78315,7 @@
         </is>
       </c>
       <c r="D1129" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G1129" t="n">
         <v>1</v>
@@ -78327,33 +78327,33 @@
         <v>2</v>
       </c>
       <c r="J1129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K1129" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="L1129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1129" t="n">
         <v>1</v>
       </c>
       <c r="N1129" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1129" t="n">
         <v>0</v>
       </c>
       <c r="P1129" t="n">
-        <v>1921990199000</v>
+        <v>1922011101000</v>
       </c>
       <c r="Q1129" t="inlineStr">
         <is>
-          <t>OUTRAS INDENIZAÇÕES - PRINC. - DEMAIS</t>
+          <t>RESTITUIÇÃO CONVÊNIOS - PRIMÁRIAS - PRINC.</t>
         </is>
       </c>
       <c r="U1129" t="n">
-        <v>2513608</v>
+        <v>27362594</v>
       </c>
       <c r="V1129" t="n">
         <v>2027</v>
@@ -78384,7 +78384,7 @@
         </is>
       </c>
       <c r="D1130" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="G1130" t="n">
         <v>1</v>
@@ -78422,7 +78422,7 @@
         </is>
       </c>
       <c r="U1130" t="n">
-        <v>27362594</v>
+        <v>502602</v>
       </c>
       <c r="V1130" t="n">
         <v>2027</v>
@@ -78453,7 +78453,7 @@
         </is>
       </c>
       <c r="D1131" t="n">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="G1131" t="n">
         <v>1</v>
@@ -78491,7 +78491,7 @@
         </is>
       </c>
       <c r="U1131" t="n">
-        <v>502602</v>
+        <v>1000</v>
       </c>
       <c r="V1131" t="n">
         <v>2027</v>
@@ -78503,7 +78503,7 @@
       </c>
       <c r="X1131" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -78522,7 +78522,7 @@
         </is>
       </c>
       <c r="D1132" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G1132" t="n">
         <v>1</v>
@@ -78537,10 +78537,10 @@
         <v>2</v>
       </c>
       <c r="K1132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L1132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M1132" t="n">
         <v>1</v>
@@ -78552,11 +78552,11 @@
         <v>0</v>
       </c>
       <c r="P1132" t="n">
-        <v>1922011101000</v>
+        <v>1922030101000</v>
       </c>
       <c r="Q1132" t="inlineStr">
         <is>
-          <t>RESTITUIÇÃO CONVÊNIOS - PRIMÁRIAS - PRINC.</t>
+          <t>RESTITUIÇÃO BENEFÍCIOS PREVIDENCIÁRIOS - PRINC. - FOLHA PAGAMENTO - INATIVOS E PENSIONISTAS</t>
         </is>
       </c>
       <c r="U1132" t="n">
@@ -78572,7 +78572,7 @@
       </c>
       <c r="X1132" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Ajusta receitas obrigatórias no GRP relacionadas à despesa de pessoal</t>
         </is>
       </c>
     </row>
@@ -78591,7 +78591,7 @@
         </is>
       </c>
       <c r="D1133" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="G1133" t="n">
         <v>1</v>
@@ -78606,30 +78606,30 @@
         <v>2</v>
       </c>
       <c r="K1133" t="n">
+        <v>6</v>
+      </c>
+      <c r="L1133" t="n">
         <v>3</v>
       </c>
-      <c r="L1133" t="n">
-        <v>0</v>
-      </c>
       <c r="M1133" t="n">
         <v>1</v>
       </c>
       <c r="N1133" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="O1133" t="n">
         <v>0</v>
       </c>
       <c r="P1133" t="n">
-        <v>1922030101000</v>
+        <v>1922063199000</v>
       </c>
       <c r="Q1133" t="inlineStr">
         <is>
-          <t>RESTITUIÇÃO BENEFÍCIOS PREVIDENCIÁRIOS - PRINC. - FOLHA PAGAMENTO - INATIVOS E PENSIONISTAS</t>
+          <t>RESTITUIÇÃO DESPESAS PRIMÁRIAS EXERCÍCIOS ANTERIORES - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1133" t="n">
-        <v>1000</v>
+        <v>653753</v>
       </c>
       <c r="V1133" t="n">
         <v>2027</v>
@@ -78641,7 +78641,7 @@
       </c>
       <c r="X1133" t="inlineStr">
         <is>
-          <t>Ajusta receitas obrigatórias no GRP relacionadas à despesa de pessoal</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -78660,7 +78660,7 @@
         </is>
       </c>
       <c r="D1134" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="G1134" t="n">
         <v>1</v>
@@ -78675,30 +78675,30 @@
         <v>2</v>
       </c>
       <c r="K1134" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="L1134" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M1134" t="n">
         <v>1</v>
       </c>
       <c r="N1134" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1134" t="n">
         <v>0</v>
       </c>
       <c r="P1134" t="n">
-        <v>1922063199000</v>
+        <v>1922520101000</v>
       </c>
       <c r="Q1134" t="inlineStr">
         <is>
-          <t>RESTITUIÇÃO DESPESAS PRIMÁRIAS EXERCÍCIOS ANTERIORES - PRINC. - DEMAIS</t>
+          <t>RESTITUIÇÃO REMUNERAÇÃO FOLHA PAGAMENTO - PESSOAL ATIVO - PRINC.</t>
         </is>
       </c>
       <c r="U1134" t="n">
-        <v>653753</v>
+        <v>1000</v>
       </c>
       <c r="V1134" t="n">
         <v>2027</v>
@@ -78710,7 +78710,7 @@
       </c>
       <c r="X1134" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Adequação das receitas de restituição - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -78729,7 +78729,7 @@
         </is>
       </c>
       <c r="D1135" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="G1135" t="n">
         <v>1</v>
@@ -78798,7 +78798,7 @@
         </is>
       </c>
       <c r="D1136" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="G1136" t="n">
         <v>1</v>
@@ -78813,7 +78813,7 @@
         <v>2</v>
       </c>
       <c r="K1136" t="n">
-        <v>52</v>
+        <v>99</v>
       </c>
       <c r="L1136" t="n">
         <v>0</v>
@@ -78828,15 +78828,15 @@
         <v>0</v>
       </c>
       <c r="P1136" t="n">
-        <v>1922520101000</v>
+        <v>1922990101000</v>
       </c>
       <c r="Q1136" t="inlineStr">
         <is>
-          <t>RESTITUIÇÃO REMUNERAÇÃO FOLHA PAGAMENTO - PESSOAL ATIVO - PRINC.</t>
+          <t>OUTRAS RESTITUIÇÕES - PRINC. - RECURSOS ORIGINÁRIOS DO FUNDO ESTADUAL DE SAÚDE - FES</t>
         </is>
       </c>
       <c r="U1136" t="n">
-        <v>1000</v>
+        <v>32626</v>
       </c>
       <c r="V1136" t="n">
         <v>2027</v>
@@ -78848,7 +78848,7 @@
       </c>
       <c r="X1136" t="inlineStr">
         <is>
-          <t>Adequação das receitas de restituição - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -78891,21 +78891,21 @@
         <v>1</v>
       </c>
       <c r="N1137" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="O1137" t="n">
         <v>0</v>
       </c>
       <c r="P1137" t="n">
-        <v>1922990101000</v>
+        <v>1922990199000</v>
       </c>
       <c r="Q1137" t="inlineStr">
         <is>
-          <t>OUTRAS RESTITUIÇÕES - PRINC. - RECURSOS ORIGINÁRIOS DO FUNDO ESTADUAL DE SAÚDE - FES</t>
+          <t>OUTRAS RESTITUIÇÕES - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1137" t="n">
-        <v>32626</v>
+        <v>258077144</v>
       </c>
       <c r="V1137" t="n">
         <v>2027</v>
@@ -78917,7 +78917,7 @@
       </c>
       <c r="X1137" t="inlineStr">
         <is>
-          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -78936,7 +78936,7 @@
         </is>
       </c>
       <c r="D1138" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G1138" t="n">
         <v>1</v>
@@ -78974,7 +78974,7 @@
         </is>
       </c>
       <c r="U1138" t="n">
-        <v>258077144</v>
+        <v>1000</v>
       </c>
       <c r="V1138" t="n">
         <v>2027</v>
@@ -78986,7 +78986,7 @@
       </c>
       <c r="X1138" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t xml:space="preserve">Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027. </t>
         </is>
       </c>
     </row>
@@ -79005,7 +79005,7 @@
         </is>
       </c>
       <c r="D1139" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G1139" t="n">
         <v>1</v>
@@ -79043,7 +79043,7 @@
         </is>
       </c>
       <c r="U1139" t="n">
-        <v>1000</v>
+        <v>1246067</v>
       </c>
       <c r="V1139" t="n">
         <v>2027</v>
@@ -79055,7 +79055,7 @@
       </c>
       <c r="X1139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027. </t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -79074,7 +79074,7 @@
         </is>
       </c>
       <c r="D1140" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G1140" t="n">
         <v>1</v>
@@ -79112,7 +79112,7 @@
         </is>
       </c>
       <c r="U1140" t="n">
-        <v>1246067</v>
+        <v>1751</v>
       </c>
       <c r="V1140" t="n">
         <v>2027</v>
@@ -79143,7 +79143,7 @@
         </is>
       </c>
       <c r="D1141" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G1141" t="n">
         <v>1</v>
@@ -79181,7 +79181,7 @@
         </is>
       </c>
       <c r="U1141" t="n">
-        <v>1751</v>
+        <v>13418</v>
       </c>
       <c r="V1141" t="n">
         <v>2027</v>
@@ -79212,7 +79212,7 @@
         </is>
       </c>
       <c r="D1142" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G1142" t="n">
         <v>1</v>
@@ -79250,7 +79250,7 @@
         </is>
       </c>
       <c r="U1142" t="n">
-        <v>13418</v>
+        <v>262703</v>
       </c>
       <c r="V1142" t="n">
         <v>2027</v>
@@ -79281,7 +79281,7 @@
         </is>
       </c>
       <c r="D1143" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G1143" t="n">
         <v>1</v>
@@ -79319,7 +79319,7 @@
         </is>
       </c>
       <c r="U1143" t="n">
-        <v>262703</v>
+        <v>92274</v>
       </c>
       <c r="V1143" t="n">
         <v>2027</v>
@@ -79350,7 +79350,7 @@
         </is>
       </c>
       <c r="D1144" t="n">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="G1144" t="n">
         <v>1</v>
@@ -79388,7 +79388,7 @@
         </is>
       </c>
       <c r="U1144" t="n">
-        <v>92274</v>
+        <v>1000</v>
       </c>
       <c r="V1144" t="n">
         <v>2027</v>
@@ -79400,7 +79400,7 @@
       </c>
       <c r="X1144" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -79419,7 +79419,7 @@
         </is>
       </c>
       <c r="D1145" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="G1145" t="n">
         <v>1</v>
@@ -79457,7 +79457,7 @@
         </is>
       </c>
       <c r="U1145" t="n">
-        <v>1000</v>
+        <v>231448</v>
       </c>
       <c r="V1145" t="n">
         <v>2027</v>
@@ -79469,7 +79469,7 @@
       </c>
       <c r="X1145" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -79488,7 +79488,7 @@
         </is>
       </c>
       <c r="D1146" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G1146" t="n">
         <v>1</v>
@@ -79526,7 +79526,7 @@
         </is>
       </c>
       <c r="U1146" t="n">
-        <v>231448</v>
+        <v>284271</v>
       </c>
       <c r="V1146" t="n">
         <v>2027</v>
@@ -79557,7 +79557,7 @@
         </is>
       </c>
       <c r="D1147" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G1147" t="n">
         <v>1</v>
@@ -79595,7 +79595,7 @@
         </is>
       </c>
       <c r="U1147" t="n">
-        <v>284271</v>
+        <v>1000</v>
       </c>
       <c r="V1147" t="n">
         <v>2027</v>
@@ -79607,7 +79607,7 @@
       </c>
       <c r="X1147" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Ajusta receitas obrigatórias no GRP relacionadas à despesa de pessoal</t>
         </is>
       </c>
     </row>
@@ -79626,7 +79626,7 @@
         </is>
       </c>
       <c r="D1148" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G1148" t="n">
         <v>1</v>
@@ -79664,7 +79664,7 @@
         </is>
       </c>
       <c r="U1148" t="n">
-        <v>1000</v>
+        <v>371822</v>
       </c>
       <c r="V1148" t="n">
         <v>2027</v>
@@ -79676,7 +79676,7 @@
       </c>
       <c r="X1148" t="inlineStr">
         <is>
-          <t>Ajusta receitas obrigatórias no GRP relacionadas à despesa de pessoal</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -79695,7 +79695,7 @@
         </is>
       </c>
       <c r="D1149" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="G1149" t="n">
         <v>1</v>
@@ -79733,7 +79733,7 @@
         </is>
       </c>
       <c r="U1149" t="n">
-        <v>371822</v>
+        <v>1000</v>
       </c>
       <c r="V1149" t="n">
         <v>2027</v>
@@ -79745,7 +79745,7 @@
       </c>
       <c r="X1149" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -79764,7 +79764,7 @@
         </is>
       </c>
       <c r="D1150" t="n">
-        <v>95</v>
+        <v>15</v>
       </c>
       <c r="G1150" t="n">
         <v>1</v>
@@ -79776,10 +79776,10 @@
         <v>2</v>
       </c>
       <c r="J1150" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K1150" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="L1150" t="n">
         <v>0</v>
@@ -79788,17 +79788,17 @@
         <v>1</v>
       </c>
       <c r="N1150" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1150" t="n">
         <v>0</v>
       </c>
       <c r="P1150" t="n">
-        <v>1922990199000</v>
+        <v>1923030101000</v>
       </c>
       <c r="Q1150" t="inlineStr">
         <is>
-          <t>OUTRAS RESTITUIÇÕES - PRINC. - DEMAIS</t>
+          <t>REVERSÃO GARANTIAS - PRINC.</t>
         </is>
       </c>
       <c r="U1150" t="n">
@@ -79842,13 +79842,13 @@
         <v>9</v>
       </c>
       <c r="I1151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J1151" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K1151" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L1151" t="n">
         <v>0</v>
@@ -79863,15 +79863,15 @@
         <v>0</v>
       </c>
       <c r="P1151" t="n">
-        <v>1923030101000</v>
+        <v>1931060101000</v>
       </c>
       <c r="Q1151" t="inlineStr">
         <is>
-          <t>REVERSÃO GARANTIAS - PRINC.</t>
+          <t>BENS DIREITOS VALORES RENÚNCIA VOLUNTÁRIA ACORDO NÃO PERSECUÇÃO PENAL - PRINC.</t>
         </is>
       </c>
       <c r="U1151" t="n">
-        <v>1000</v>
+        <v>680555</v>
       </c>
       <c r="V1151" t="n">
         <v>2027</v>
@@ -79883,7 +79883,7 @@
       </c>
       <c r="X1151" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -79902,7 +79902,7 @@
         </is>
       </c>
       <c r="D1152" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G1152" t="n">
         <v>1</v>
@@ -79911,36 +79911,36 @@
         <v>9</v>
       </c>
       <c r="I1152" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J1152" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K1152" t="n">
-        <v>6</v>
+        <v>99</v>
       </c>
       <c r="L1152" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M1152" t="n">
         <v>1</v>
       </c>
       <c r="N1152" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="O1152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P1152" t="n">
-        <v>1931060101000</v>
+        <v>1999992108001</v>
       </c>
       <c r="Q1152" t="inlineStr">
         <is>
-          <t>BENS DIREITOS VALORES RENÚNCIA VOLUNTÁRIA ACORDO NÃO PERSECUÇÃO PENAL - PRINC.</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - RECEITAS ADICIONAIS À CONCESSÃO - PPP - AEROPORTUÁRIA</t>
         </is>
       </c>
       <c r="U1152" t="n">
-        <v>680555</v>
+        <v>311572</v>
       </c>
       <c r="V1152" t="n">
         <v>2027</v>
@@ -79952,7 +79952,7 @@
       </c>
       <c r="X1152" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
         </is>
       </c>
     </row>
@@ -79971,7 +79971,7 @@
         </is>
       </c>
       <c r="D1153" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G1153" t="n">
         <v>1</v>
@@ -80009,7 +80009,7 @@
         </is>
       </c>
       <c r="U1153" t="n">
-        <v>311572</v>
+        <v>4955097</v>
       </c>
       <c r="V1153" t="n">
         <v>2027</v>
@@ -80021,7 +80021,7 @@
       </c>
       <c r="X1153" t="inlineStr">
         <is>
-          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
+          <t>Foi utilizado como parâmetro o último valor de receita compartilhada efetivamente pago pela Concessionária, sendo o mesmo atualizado pelo IPCA projetado para os anos seguintes.</t>
         </is>
       </c>
     </row>
@@ -80067,18 +80067,18 @@
         <v>8</v>
       </c>
       <c r="O1154" t="n">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="P1154" t="n">
-        <v>1999992108001</v>
+        <v>1999992108999</v>
       </c>
       <c r="Q1154" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - RECEITAS ADICIONAIS À CONCESSÃO - PPP - AEROPORTUÁRIA</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - RECEITAS ADICIONAIS À CONCESSÃO - PPP - OUTROS</t>
         </is>
       </c>
       <c r="U1154" t="n">
-        <v>4955097</v>
+        <v>7846113</v>
       </c>
       <c r="V1154" t="n">
         <v>2027</v>
@@ -80090,7 +80090,7 @@
       </c>
       <c r="X1154" t="inlineStr">
         <is>
-          <t>Foi utilizado como parâmetro o último valor de receita compartilhada efetivamente pago pela Concessionária, sendo o mesmo atualizado pelo IPCA projetado para os anos seguintes.</t>
+          <t xml:space="preserve">Foi utilizado como parâmetro o último valor de receita compartilhada efetivamente pago pela Concessionária, sendo o mesmo atualizado pelo IPCA projetado para os anos seguintes. </t>
         </is>
       </c>
     </row>
@@ -80133,21 +80133,21 @@
         <v>1</v>
       </c>
       <c r="N1155" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O1155" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="P1155" t="n">
-        <v>1999992108999</v>
+        <v>1999992111000</v>
       </c>
       <c r="Q1155" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - RECEITAS ADICIONAIS À CONCESSÃO - PPP - OUTROS</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - BANCO DO ESTADO DE MINAS GERAIS - BEMGE</t>
         </is>
       </c>
       <c r="U1155" t="n">
-        <v>7846113</v>
+        <v>2600000</v>
       </c>
       <c r="V1155" t="n">
         <v>2027</v>
@@ -80159,7 +80159,7 @@
       </c>
       <c r="X1155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Foi utilizado como parâmetro o último valor de receita compartilhada efetivamente pago pela Concessionária, sendo o mesmo atualizado pelo IPCA projetado para os anos seguintes. </t>
+          <t>Calculou-se a média de repasse dos últimos 4 anos, desconsiderando o repasse do precatório ocorrido em 2023.</t>
         </is>
       </c>
     </row>
@@ -80202,21 +80202,21 @@
         <v>1</v>
       </c>
       <c r="N1156" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="O1156" t="n">
         <v>0</v>
       </c>
       <c r="P1156" t="n">
-        <v>1999992111000</v>
+        <v>1999992115000</v>
       </c>
       <c r="Q1156" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - BANCO DO ESTADO DE MINAS GERAIS - BEMGE</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - GESTÃO DE VEÍCULOS APREENDIDOS E REMOVIDOS</t>
         </is>
       </c>
       <c r="U1156" t="n">
-        <v>2600000</v>
+        <v>144542903</v>
       </c>
       <c r="V1156" t="n">
         <v>2027</v>
@@ -80228,7 +80228,7 @@
       </c>
       <c r="X1156" t="inlineStr">
         <is>
-          <t>Calculou-se a média de repasse dos últimos 4 anos, desconsiderando o repasse do precatório ocorrido em 2023.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -80271,21 +80271,21 @@
         <v>1</v>
       </c>
       <c r="N1157" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="O1157" t="n">
         <v>0</v>
       </c>
       <c r="P1157" t="n">
-        <v>1999992115000</v>
+        <v>1999992117000</v>
       </c>
       <c r="Q1157" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - GESTÃO DE VEÍCULOS APREENDIDOS E REMOVIDOS</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - BENS, DIREITOS E VALORES OBJETO DE RENÚNCIA VOLUNTÁRIA EM ACORDO DE NÃO PERSECUÇÃO CÍVEL</t>
         </is>
       </c>
       <c r="U1157" t="n">
-        <v>144542903</v>
+        <v>111144</v>
       </c>
       <c r="V1157" t="n">
         <v>2027</v>
@@ -80316,7 +80316,7 @@
         </is>
       </c>
       <c r="D1158" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G1158" t="n">
         <v>1</v>
@@ -80340,21 +80340,21 @@
         <v>1</v>
       </c>
       <c r="N1158" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="O1158" t="n">
         <v>0</v>
       </c>
       <c r="P1158" t="n">
-        <v>1999992117000</v>
+        <v>1999992199000</v>
       </c>
       <c r="Q1158" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - BENS, DIREITOS E VALORES OBJETO DE RENÚNCIA VOLUNTÁRIA EM ACORDO DE NÃO PERSECUÇÃO CÍVEL</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1158" t="n">
-        <v>111144</v>
+        <v>13285715</v>
       </c>
       <c r="V1158" t="n">
         <v>2027</v>
@@ -80366,7 +80366,7 @@
       </c>
       <c r="X1158" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
         </is>
       </c>
     </row>
@@ -80385,7 +80385,7 @@
         </is>
       </c>
       <c r="D1159" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G1159" t="n">
         <v>1</v>
@@ -80423,7 +80423,7 @@
         </is>
       </c>
       <c r="U1159" t="n">
-        <v>13285715</v>
+        <v>43198510</v>
       </c>
       <c r="V1159" t="n">
         <v>2027</v>
@@ -80435,7 +80435,7 @@
       </c>
       <c r="X1159" t="inlineStr">
         <is>
-          <t>APLICAÇÃO DO PERCENTUAL DE DESVINCULAÇÃO PREVISTO NO ARTIGO 76-A DO ATO DAS DISPOSIÇÕES CONSTITUCIONAIS TRANSITÓRIAS (ADCT) SOBRE AS RECEITAS ESTADUAIS PASSÍVEIS DE DESVINCULAÇÃO ATÉ 2032</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -80475,7 +80475,7 @@
         <v>2</v>
       </c>
       <c r="M1160" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1160" t="n">
         <v>99</v>
@@ -80484,15 +80484,15 @@
         <v>0</v>
       </c>
       <c r="P1160" t="n">
-        <v>1999992199000</v>
+        <v>1999992299000</v>
       </c>
       <c r="Q1160" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - PRINC. - DEMAIS</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - MJM - DEMAIS</t>
         </is>
       </c>
       <c r="U1160" t="n">
-        <v>43198510</v>
+        <v>747071</v>
       </c>
       <c r="V1160" t="n">
         <v>2027</v>
@@ -80544,7 +80544,7 @@
         <v>2</v>
       </c>
       <c r="M1161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1161" t="n">
         <v>99</v>
@@ -80553,15 +80553,15 @@
         <v>0</v>
       </c>
       <c r="P1161" t="n">
-        <v>1999992299000</v>
+        <v>1999992399000</v>
       </c>
       <c r="Q1161" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - MJM - DEMAIS</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - DA - DEMAIS</t>
         </is>
       </c>
       <c r="U1161" t="n">
-        <v>747071</v>
+        <v>1000</v>
       </c>
       <c r="V1161" t="n">
         <v>2027</v>
@@ -80573,7 +80573,7 @@
       </c>
       <c r="X1161" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
         </is>
       </c>
     </row>
@@ -80613,7 +80613,7 @@
         <v>2</v>
       </c>
       <c r="M1162" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N1162" t="n">
         <v>99</v>
@@ -80622,15 +80622,15 @@
         <v>0</v>
       </c>
       <c r="P1162" t="n">
-        <v>1999992399000</v>
+        <v>1999992499000</v>
       </c>
       <c r="Q1162" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - DA - DEMAIS</t>
+          <t>OUTRAS REC. - PRIMÁRIAS - DA-MJM - DEMAIS</t>
         </is>
       </c>
       <c r="U1162" t="n">
-        <v>1000</v>
+        <v>100801</v>
       </c>
       <c r="V1162" t="n">
         <v>2027</v>
@@ -80642,7 +80642,7 @@
       </c>
       <c r="X1162" t="inlineStr">
         <is>
-          <t>Em virtude da complexidade na projeção do fluxo de arrecadação, optou-se pelo lançamento de valor estimado de R$ 1.000 na LDO 2027.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -80661,45 +80661,45 @@
         </is>
       </c>
       <c r="D1163" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G1163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H1163" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I1163" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J1163" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K1163" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="L1163" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M1163" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N1163" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1163" t="n">
         <v>0</v>
       </c>
       <c r="P1163" t="n">
-        <v>1999992499000</v>
+        <v>2213010101000</v>
       </c>
       <c r="Q1163" t="inlineStr">
         <is>
-          <t>OUTRAS REC. - PRIMÁRIAS - DA-MJM - DEMAIS</t>
+          <t>ALIENAÇÃO BENS MÓVEIS SEMOVENTES - PRINC.</t>
         </is>
       </c>
       <c r="U1163" t="n">
-        <v>100801</v>
+        <v>18727763</v>
       </c>
       <c r="V1163" t="n">
         <v>2027</v>
@@ -80739,10 +80739,10 @@
         <v>2</v>
       </c>
       <c r="I1164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J1164" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K1164" t="n">
         <v>1</v>
@@ -80760,15 +80760,15 @@
         <v>0</v>
       </c>
       <c r="P1164" t="n">
-        <v>2213010101000</v>
+        <v>2221010101000</v>
       </c>
       <c r="Q1164" t="inlineStr">
         <is>
-          <t>ALIENAÇÃO BENS MÓVEIS SEMOVENTES - PRINC.</t>
+          <t>ALIENAÇÃO BENS IMÓVEIS - PRINC.</t>
         </is>
       </c>
       <c r="U1164" t="n">
-        <v>18727763</v>
+        <v>8600000</v>
       </c>
       <c r="V1164" t="n">
         <v>2027</v>
@@ -80780,7 +80780,7 @@
       </c>
       <c r="X1164" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>Os valores previstos se basearão somente no valor alienado em 2025, podendo sofrer alterações.</t>
         </is>
       </c>
     </row>
@@ -80799,22 +80799,22 @@
         </is>
       </c>
       <c r="D1165" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="G1165" t="n">
         <v>2</v>
       </c>
       <c r="H1165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I1165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J1165" t="n">
         <v>1</v>
       </c>
       <c r="K1165" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L1165" t="n">
         <v>0</v>
@@ -80829,15 +80829,15 @@
         <v>0</v>
       </c>
       <c r="P1165" t="n">
-        <v>2221010101000</v>
+        <v>2311060101000</v>
       </c>
       <c r="Q1165" t="inlineStr">
         <is>
-          <t>ALIENAÇÃO BENS IMÓVEIS - PRINC.</t>
+          <t>AMORTIZAÇÃO EMPRÉSTIMOS CONTRATUAIS - PRINC.</t>
         </is>
       </c>
       <c r="U1165" t="n">
-        <v>8600000</v>
+        <v>798202</v>
       </c>
       <c r="V1165" t="n">
         <v>2027</v>
@@ -80849,7 +80849,7 @@
       </c>
       <c r="X1165" t="inlineStr">
         <is>
-          <t>Os valores previstos se basearão somente no valor alienado em 2025, podendo sofrer alterações.</t>
+          <t>Foi utilizada a previsão para 2026, amortizada em 5% para o exercício de 2027.</t>
         </is>
       </c>
     </row>
@@ -80868,7 +80868,7 @@
         </is>
       </c>
       <c r="D1166" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G1166" t="n">
         <v>2</v>
@@ -80883,30 +80883,30 @@
         <v>1</v>
       </c>
       <c r="K1166" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L1166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1166" t="n">
         <v>1</v>
       </c>
       <c r="N1166" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="O1166" t="n">
         <v>0</v>
       </c>
       <c r="P1166" t="n">
-        <v>2311060101000</v>
+        <v>2311071199000</v>
       </c>
       <c r="Q1166" t="inlineStr">
         <is>
-          <t>AMORTIZAÇÃO EMPRÉSTIMOS CONTRATUAIS - PRINC.</t>
+          <t>AMORTIZAÇÃO FINANCIAMENTOS GERAL - PRINC. - DEMAIS</t>
         </is>
       </c>
       <c r="U1166" t="n">
-        <v>798202</v>
+        <v>171671</v>
       </c>
       <c r="V1166" t="n">
         <v>2027</v>
@@ -80918,7 +80918,7 @@
       </c>
       <c r="X1166" t="inlineStr">
         <is>
-          <t>Foi utilizada a previsão para 2026, amortizada em 5% para o exercício de 2027.</t>
+          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
         </is>
       </c>
     </row>
@@ -80937,45 +80937,45 @@
         </is>
       </c>
       <c r="D1167" t="n">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="G1167" t="n">
         <v>2</v>
       </c>
       <c r="H1167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I1167" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J1167" t="n">
         <v>1</v>
       </c>
       <c r="K1167" t="n">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="L1167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M1167" t="n">
         <v>1</v>
       </c>
       <c r="N1167" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="O1167" t="n">
         <v>0</v>
       </c>
       <c r="P1167" t="n">
-        <v>2311071199000</v>
+        <v>2441520101000</v>
       </c>
       <c r="Q1167" t="inlineStr">
         <is>
-          <t>AMORTIZAÇÃO FINANCIAMENTOS GERAL - PRINC. - DEMAIS</t>
+          <t>TRANSF. FEF - LC N° 212/2025 - PRINC.</t>
         </is>
       </c>
       <c r="U1167" t="n">
-        <v>171671</v>
+        <v>386591331</v>
       </c>
       <c r="V1167" t="n">
         <v>2027</v>
@@ -80987,7 +80987,7 @@
       </c>
       <c r="X1167" t="inlineStr">
         <is>
-          <t>Foi utilizada a receita prevista para 2026 corrigida para 2027 pelo PIB e IPCA.</t>
+          <t>No momento atual, diante da indisponibilidade de informações consolidadas dos demais estados ¿ especialmente no que se refere às projeções de dívida, Receita Corrente Líquida (RCL) e coeficientes do Fundo de Participação dos Estados (FPE), que impactam diretamente a distribuição dos recursos do Fundo de Equalização Federativa (FEF) ¿ e considerando, ainda, que os entes federativos se encontram em diferentes estágios do processo de adesão ao Programa de Pleno Pagamento de Dívidas dos Estados (PROPAG), torna-se inviável a elaboração de uma estimativa mais robusta e factível da receita a ser auferida por meio desse mecanismo.</t>
         </is>
       </c>
     </row>
@@ -81006,45 +81006,45 @@
         </is>
       </c>
       <c r="D1168" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G1168" t="n">
         <v>2</v>
       </c>
       <c r="H1168" t="n">
+        <v>9</v>
+      </c>
+      <c r="I1168" t="n">
+        <v>9</v>
+      </c>
+      <c r="J1168" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1168" t="n">
+        <v>99</v>
+      </c>
+      <c r="L1168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1168" t="n">
+        <v>1</v>
+      </c>
+      <c r="N1168" t="n">
         <v>4</v>
       </c>
-      <c r="I1168" t="n">
-        <v>4</v>
-      </c>
-      <c r="J1168" t="n">
-        <v>1</v>
-      </c>
-      <c r="K1168" t="n">
-        <v>52</v>
-      </c>
-      <c r="L1168" t="n">
-        <v>0</v>
-      </c>
-      <c r="M1168" t="n">
-        <v>1</v>
-      </c>
-      <c r="N1168" t="n">
-        <v>1</v>
-      </c>
       <c r="O1168" t="n">
         <v>0</v>
       </c>
       <c r="P1168" t="n">
-        <v>2441520101000</v>
+        <v>2999990104000</v>
       </c>
       <c r="Q1168" t="inlineStr">
         <is>
-          <t>TRANSF. FEF - LC N° 212/2025 - PRINC.</t>
+          <t>DEMAIS REC. CAPITAL - PRINC. - ROMPIMENTO DA BARRAGEM DE FUNDÃO EM MARIANA - ACORDO JUDICIAL DE REPARAÇÃO INTEGRAL E DEFINITIVA</t>
         </is>
       </c>
       <c r="U1168" t="n">
-        <v>386591331</v>
+        <v>778348874</v>
       </c>
       <c r="V1168" t="n">
         <v>2027</v>
@@ -81056,7 +81056,7 @@
       </c>
       <c r="X1168" t="inlineStr">
         <is>
-          <t>No momento atual, diante da indisponibilidade de informações consolidadas dos demais estados ¿ especialmente no que se refere às projeções de dívida, Receita Corrente Líquida (RCL) e coeficientes do Fundo de Participação dos Estados (FPE), que impactam diretamente a distribuição dos recursos do Fundo de Equalização Federativa (FEF) ¿ e considerando, ainda, que os entes federativos se encontram em diferentes estágios do processo de adesão ao Programa de Pleno Pagamento de Dívidas dos Estados (PROPAG), torna-se inviável a elaboração de uma estimativa mais robusta e factível da receita a ser auferida por meio desse mecanismo.</t>
+          <t>Receita com previsão enviada pela Secretaria de Estado de Planejamento e Gestão.</t>
         </is>
       </c>
     </row>
@@ -81075,16 +81075,16 @@
         </is>
       </c>
       <c r="D1169" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G1169" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H1169" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I1169" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J1169" t="n">
         <v>9</v>
@@ -81093,27 +81093,27 @@
         <v>99</v>
       </c>
       <c r="L1169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1169" t="n">
         <v>1</v>
       </c>
       <c r="N1169" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O1169" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="P1169" t="n">
-        <v>2999990104000</v>
+        <v>7219991110051</v>
       </c>
       <c r="Q1169" t="inlineStr">
         <is>
-          <t>DEMAIS REC. CAPITAL - PRINC. - ROMPIMENTO DA BARRAGEM DE FUNDÃO EM MARIANA - ACORDO JUDICIAL DE REPARAÇÃO INTEGRAL E DEFINITIVA</t>
+          <t>REC. INTRA. - DEMAIS CONTRIB. SOC. - PRINC. - CONTRIB. PATRONAL MILITAR APOSENTADORIA - ATIVO</t>
         </is>
       </c>
       <c r="U1169" t="n">
-        <v>778348874</v>
+        <v>257524180</v>
       </c>
       <c r="V1169" t="n">
         <v>2027</v>
@@ -81125,7 +81125,7 @@
       </c>
       <c r="X1169" t="inlineStr">
         <is>
-          <t>Receita com previsão enviada pela Secretaria de Estado de Planejamento e Gestão.</t>
+          <t>RECEITA DE CONTRIBUIÇÕES: PROJEÇÃO COM BASE NA RECEITA EXECUTADA ATÉ MARÇO DE 2025, INCORPORANDO CRESCIMENTO VEGETATIVO, REAJUSTES E OUTROS IMPACTOS.</t>
         </is>
       </c>
     </row>
@@ -81171,18 +81171,18 @@
         <v>10</v>
       </c>
       <c r="O1170" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P1170" t="n">
-        <v>7219991110051</v>
+        <v>7219991110052</v>
       </c>
       <c r="Q1170" t="inlineStr">
         <is>
-          <t>REC. INTRA. - DEMAIS CONTRIB. SOC. - PRINC. - CONTRIB. PATRONAL MILITAR APOSENTADORIA - ATIVO</t>
+          <t>REC. INTRA. - DEMAIS CONTRIB. SOC. - PRINC. - CONTRIB. PATRONAL MILITAR APOSENTADORIA - INATIVO</t>
         </is>
       </c>
       <c r="U1170" t="n">
-        <v>257524180</v>
+        <v>390963136</v>
       </c>
       <c r="V1170" t="n">
         <v>2027</v>
@@ -81213,45 +81213,45 @@
         </is>
       </c>
       <c r="D1171" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="G1171" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H1171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I1171" t="n">
         <v>1</v>
       </c>
       <c r="J1171" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K1171" t="n">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="L1171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M1171" t="n">
         <v>1</v>
       </c>
       <c r="N1171" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O1171" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="P1171" t="n">
-        <v>7219991110052</v>
+        <v>9112510102000</v>
       </c>
       <c r="Q1171" t="inlineStr">
         <is>
-          <t>REC. INTRA. - DEMAIS CONTRIB. SOC. - PRINC. - CONTRIB. PATRONAL MILITAR APOSENTADORIA - INATIVO</t>
+          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1171" t="n">
-        <v>390963136</v>
+        <v>-6730265620</v>
       </c>
       <c r="V1171" t="n">
         <v>2027</v>
@@ -81263,7 +81263,7 @@
       </c>
       <c r="X1171" t="inlineStr">
         <is>
-          <t>RECEITA DE CONTRIBUIÇÕES: PROJEÇÃO COM BASE NA RECEITA EXECUTADA ATÉ MARÇO DE 2025, INCORPORANDO CRESCIMENTO VEGETATIVO, REAJUSTES E OUTROS IMPACTOS.</t>
+          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81282,7 +81282,7 @@
         </is>
       </c>
       <c r="D1172" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1172" t="n">
         <v>9</v>
@@ -81306,21 +81306,21 @@
         <v>1</v>
       </c>
       <c r="N1172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1172" t="n">
         <v>0</v>
       </c>
       <c r="P1172" t="n">
-        <v>9112510102000</v>
+        <v>9112510103000</v>
       </c>
       <c r="Q1172" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1172" t="n">
-        <v>-6730265620</v>
+        <v>-1346053124</v>
       </c>
       <c r="V1172" t="n">
         <v>2027</v>
@@ -81332,7 +81332,7 @@
       </c>
       <c r="X1172" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81351,7 +81351,7 @@
         </is>
       </c>
       <c r="D1173" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1173" t="n">
         <v>9</v>
@@ -81372,24 +81372,24 @@
         <v>0</v>
       </c>
       <c r="M1173" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1173" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1173" t="n">
         <v>0</v>
       </c>
       <c r="P1173" t="n">
-        <v>9112510103000</v>
+        <v>9112510202000</v>
       </c>
       <c r="Q1173" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1173" t="n">
-        <v>-1346053124</v>
+        <v>-440382545</v>
       </c>
       <c r="V1173" t="n">
         <v>2027</v>
@@ -81401,7 +81401,7 @@
       </c>
       <c r="X1173" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81420,7 +81420,7 @@
         </is>
       </c>
       <c r="D1174" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1174" t="n">
         <v>9</v>
@@ -81444,21 +81444,21 @@
         <v>2</v>
       </c>
       <c r="N1174" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1174" t="n">
         <v>0</v>
       </c>
       <c r="P1174" t="n">
-        <v>9112510202000</v>
+        <v>9112510203000</v>
       </c>
       <c r="Q1174" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1174" t="n">
-        <v>-440382545</v>
+        <v>-88076509</v>
       </c>
       <c r="V1174" t="n">
         <v>2027</v>
@@ -81470,7 +81470,7 @@
       </c>
       <c r="X1174" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81489,7 +81489,7 @@
         </is>
       </c>
       <c r="D1175" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1175" t="n">
         <v>9</v>
@@ -81510,24 +81510,24 @@
         <v>0</v>
       </c>
       <c r="M1175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1175" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1175" t="n">
         <v>0</v>
       </c>
       <c r="P1175" t="n">
-        <v>9112510203000</v>
+        <v>9112510302000</v>
       </c>
       <c r="Q1175" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1175" t="n">
-        <v>-88076509</v>
+        <v>-176418275</v>
       </c>
       <c r="V1175" t="n">
         <v>2027</v>
@@ -81539,7 +81539,7 @@
       </c>
       <c r="X1175" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81558,7 +81558,7 @@
         </is>
       </c>
       <c r="D1176" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1176" t="n">
         <v>9</v>
@@ -81582,21 +81582,21 @@
         <v>3</v>
       </c>
       <c r="N1176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1176" t="n">
         <v>0</v>
       </c>
       <c r="P1176" t="n">
-        <v>9112510302000</v>
+        <v>9112510303000</v>
       </c>
       <c r="Q1176" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1176" t="n">
-        <v>-176418275</v>
+        <v>-35283655</v>
       </c>
       <c r="V1176" t="n">
         <v>2027</v>
@@ -81608,7 +81608,7 @@
       </c>
       <c r="X1176" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81642,30 +81642,30 @@
         <v>2</v>
       </c>
       <c r="K1177" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L1177" t="n">
         <v>0</v>
       </c>
       <c r="M1177" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1177" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1177" t="n">
         <v>0</v>
       </c>
       <c r="P1177" t="n">
-        <v>9112510303000</v>
+        <v>9112520102000</v>
       </c>
       <c r="Q1177" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - IPVA - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1177" t="n">
-        <v>-35283655</v>
+        <v>-469496703</v>
       </c>
       <c r="V1177" t="n">
         <v>2027</v>
@@ -81677,7 +81677,7 @@
       </c>
       <c r="X1177" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - IPVA - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81717,7 +81717,7 @@
         <v>0</v>
       </c>
       <c r="M1178" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1178" t="n">
         <v>2</v>
@@ -81726,15 +81726,15 @@
         <v>0</v>
       </c>
       <c r="P1178" t="n">
-        <v>9112520102000</v>
+        <v>9112520202000</v>
       </c>
       <c r="Q1178" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1178" t="n">
-        <v>-469496703</v>
+        <v>-39568452</v>
       </c>
       <c r="V1178" t="n">
         <v>2027</v>
@@ -81746,7 +81746,7 @@
       </c>
       <c r="X1178" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81786,7 +81786,7 @@
         <v>0</v>
       </c>
       <c r="M1179" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1179" t="n">
         <v>2</v>
@@ -81795,15 +81795,15 @@
         <v>0</v>
       </c>
       <c r="P1179" t="n">
-        <v>9112520202000</v>
+        <v>9112520302000</v>
       </c>
       <c r="Q1179" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ITCD - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1179" t="n">
-        <v>-39568452</v>
+        <v>-6352385</v>
       </c>
       <c r="V1179" t="n">
         <v>2027</v>
@@ -81815,7 +81815,7 @@
       </c>
       <c r="X1179" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de Dedução Rec. - ITCD - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -81834,7 +81834,7 @@
         </is>
       </c>
       <c r="D1180" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1180" t="n">
         <v>9</v>
@@ -81846,33 +81846,33 @@
         <v>1</v>
       </c>
       <c r="J1180" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K1180" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L1180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M1180" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1180" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O1180" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1180" t="n">
-        <v>9112520302000</v>
+        <v>9114501101002</v>
       </c>
       <c r="Q1180" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ITCD - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1180" t="n">
-        <v>-6352385</v>
+        <v>-328488</v>
       </c>
       <c r="V1180" t="n">
         <v>2027</v>
@@ -81884,7 +81884,7 @@
       </c>
       <c r="X1180" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ITCD - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -81903,7 +81903,7 @@
         </is>
       </c>
       <c r="D1181" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1181" t="n">
         <v>9</v>
@@ -81927,21 +81927,21 @@
         <v>1</v>
       </c>
       <c r="N1181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1181" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1181" t="n">
-        <v>9114501101002</v>
+        <v>9114501102000</v>
       </c>
       <c r="Q1181" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1181" t="n">
-        <v>-328488</v>
+        <v>-23077484102</v>
       </c>
       <c r="V1181" t="n">
         <v>2027</v>
@@ -81953,7 +81953,7 @@
       </c>
       <c r="X1181" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -81972,7 +81972,7 @@
         </is>
       </c>
       <c r="D1182" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1182" t="n">
         <v>9</v>
@@ -81996,21 +81996,21 @@
         <v>1</v>
       </c>
       <c r="N1182" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1182" t="n">
         <v>0</v>
       </c>
       <c r="P1182" t="n">
-        <v>9114501102000</v>
+        <v>9114501103000</v>
       </c>
       <c r="Q1182" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1182" t="n">
-        <v>-23077484102</v>
+        <v>-13846490461</v>
       </c>
       <c r="V1182" t="n">
         <v>2027</v>
@@ -82022,7 +82022,7 @@
       </c>
       <c r="X1182" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82041,7 +82041,7 @@
         </is>
       </c>
       <c r="D1183" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1183" t="n">
         <v>9</v>
@@ -82062,24 +82062,24 @@
         <v>1</v>
       </c>
       <c r="M1183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N1183" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O1183" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1183" t="n">
-        <v>9114501103000</v>
+        <v>9114501201002</v>
       </c>
       <c r="Q1183" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1183" t="n">
-        <v>-13846490461</v>
+        <v>-638942</v>
       </c>
       <c r="V1183" t="n">
         <v>2027</v>
@@ -82091,7 +82091,7 @@
       </c>
       <c r="X1183" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - Princ. - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -82110,7 +82110,7 @@
         </is>
       </c>
       <c r="D1184" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1184" t="n">
         <v>9</v>
@@ -82134,21 +82134,21 @@
         <v>2</v>
       </c>
       <c r="N1184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1184" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1184" t="n">
-        <v>9114501201002</v>
+        <v>9114501202000</v>
       </c>
       <c r="Q1184" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1184" t="n">
-        <v>-638942</v>
+        <v>-255087472</v>
       </c>
       <c r="V1184" t="n">
         <v>2027</v>
@@ -82160,7 +82160,7 @@
       </c>
       <c r="X1184" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - MJM - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -82179,7 +82179,7 @@
         </is>
       </c>
       <c r="D1185" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1185" t="n">
         <v>9</v>
@@ -82203,21 +82203,21 @@
         <v>2</v>
       </c>
       <c r="N1185" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1185" t="n">
         <v>0</v>
       </c>
       <c r="P1185" t="n">
-        <v>9114501202000</v>
+        <v>9114501203000</v>
       </c>
       <c r="Q1185" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1185" t="n">
-        <v>-255087472</v>
+        <v>-153052483</v>
       </c>
       <c r="V1185" t="n">
         <v>2027</v>
@@ -82229,7 +82229,7 @@
       </c>
       <c r="X1185" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82248,7 +82248,7 @@
         </is>
       </c>
       <c r="D1186" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G1186" t="n">
         <v>9</v>
@@ -82269,24 +82269,24 @@
         <v>1</v>
       </c>
       <c r="M1186" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N1186" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O1186" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P1186" t="n">
-        <v>9114501203000</v>
+        <v>9114501301002</v>
       </c>
       <c r="Q1186" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - MJM - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
         </is>
       </c>
       <c r="U1186" t="n">
-        <v>-153052483</v>
+        <v>-7869701</v>
       </c>
       <c r="V1186" t="n">
         <v>2027</v>
@@ -82298,7 +82298,7 @@
       </c>
       <c r="X1186" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - MJM - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receita de DEDUCAO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
         </is>
       </c>
     </row>
@@ -82317,7 +82317,7 @@
         </is>
       </c>
       <c r="D1187" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G1187" t="n">
         <v>9</v>
@@ -82341,21 +82341,21 @@
         <v>3</v>
       </c>
       <c r="N1187" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O1187" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P1187" t="n">
-        <v>9114501301002</v>
+        <v>9114501302000</v>
       </c>
       <c r="Q1187" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSÃO DE DIREITOS CREDITÓRIOS - LEI ESTADUAL Nº 19.266/10</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1187" t="n">
-        <v>-7869701</v>
+        <v>-201596219</v>
       </c>
       <c r="V1187" t="n">
         <v>2027</v>
@@ -82367,7 +82367,7 @@
       </c>
       <c r="X1187" t="inlineStr">
         <is>
-          <t>Receita de DEDUCAO REC. - ICMS - DA - COTA PARTE DO ESTADO - CESSAO DE DIREITOS CREDITORIOS - LEI ESTADUAL NO 19.266/10</t>
+          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte dos Municípios</t>
         </is>
       </c>
     </row>
@@ -82386,7 +82386,7 @@
         </is>
       </c>
       <c r="D1188" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1188" t="n">
         <v>9</v>
@@ -82410,21 +82410,21 @@
         <v>3</v>
       </c>
       <c r="N1188" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1188" t="n">
         <v>0</v>
       </c>
       <c r="P1188" t="n">
-        <v>9114501302000</v>
+        <v>9114501303000</v>
       </c>
       <c r="Q1188" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1188" t="n">
-        <v>-201596219</v>
+        <v>-120957732</v>
       </c>
       <c r="V1188" t="n">
         <v>2027</v>
@@ -82436,7 +82436,7 @@
       </c>
       <c r="X1188" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte dos Municípios</t>
+          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte do Estado para o FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82473,27 +82473,27 @@
         <v>50</v>
       </c>
       <c r="L1189" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M1189" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N1189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1189" t="n">
         <v>0</v>
       </c>
       <c r="P1189" t="n">
-        <v>9114501303000</v>
+        <v>9114502102000</v>
       </c>
       <c r="Q1189" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ICMS - DA - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>DEDUÇÃO REC. - ADICIONAL ICMS - FEM - PRINC. - COTA PARTE DO FUNDEB</t>
         </is>
       </c>
       <c r="U1189" t="n">
-        <v>-120957732</v>
+        <v>-224000000</v>
       </c>
       <c r="V1189" t="n">
         <v>2027</v>
@@ -82505,7 +82505,7 @@
       </c>
       <c r="X1189" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - ICMS - DA - Cota Parte do Estado para o FUNDEB</t>
+          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -82524,7 +82524,7 @@
         </is>
       </c>
       <c r="D1190" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1190" t="n">
         <v>9</v>
@@ -82536,13 +82536,13 @@
         <v>1</v>
       </c>
       <c r="J1190" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K1190" t="n">
         <v>50</v>
       </c>
       <c r="L1190" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M1190" t="n">
         <v>1</v>
@@ -82554,15 +82554,15 @@
         <v>0</v>
       </c>
       <c r="P1190" t="n">
-        <v>9114502102000</v>
+        <v>9116500102000</v>
       </c>
       <c r="Q1190" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - ADICIONAL ICMS - FEM - PRINC. - COTA PARTE DO FUNDEB</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1190" t="n">
-        <v>-224000000</v>
+        <v>-64413502</v>
       </c>
       <c r="V1190" t="n">
         <v>2027</v>
@@ -82574,7 +82574,7 @@
       </c>
       <c r="X1190" t="inlineStr">
         <is>
-          <t>Receitas SEF - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Inclui IBS - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
         </is>
       </c>
     </row>
@@ -82593,7 +82593,7 @@
         </is>
       </c>
       <c r="D1191" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1191" t="n">
         <v>9</v>
@@ -82617,21 +82617,21 @@
         <v>1</v>
       </c>
       <c r="N1191" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1191" t="n">
         <v>0</v>
       </c>
       <c r="P1191" t="n">
-        <v>9116500102000</v>
+        <v>9116500103000</v>
       </c>
       <c r="Q1191" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DOS MUNICÍPIOS</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
         </is>
       </c>
       <c r="U1191" t="n">
-        <v>-64413502</v>
+        <v>-38648102</v>
       </c>
       <c r="V1191" t="n">
         <v>2027</v>
@@ -82662,7 +82662,7 @@
         </is>
       </c>
       <c r="D1192" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1192" t="n">
         <v>9</v>
@@ -82686,21 +82686,21 @@
         <v>1</v>
       </c>
       <c r="N1192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O1192" t="n">
         <v>0</v>
       </c>
       <c r="P1192" t="n">
-        <v>9116500103000</v>
+        <v>9116500104000</v>
       </c>
       <c r="Q1192" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O FUNDEB</t>
+          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O COMITÊ GESTOR DO IBS</t>
         </is>
       </c>
       <c r="U1192" t="n">
-        <v>-38648102</v>
+        <v>-96620253</v>
       </c>
       <c r="V1192" t="n">
         <v>2027</v>
@@ -82731,19 +82731,19 @@
         </is>
       </c>
       <c r="D1193" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1193" t="n">
         <v>9</v>
       </c>
       <c r="H1193" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I1193" t="n">
         <v>1</v>
       </c>
       <c r="J1193" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K1193" t="n">
         <v>50</v>
@@ -82755,21 +82755,21 @@
         <v>1</v>
       </c>
       <c r="N1193" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O1193" t="n">
         <v>0</v>
       </c>
       <c r="P1193" t="n">
-        <v>9116500104000</v>
+        <v>9711500102000</v>
       </c>
       <c r="Q1193" t="inlineStr">
         <is>
-          <t>IBS ESTADO - PRINC. - COTA PARTE DO ESTADO PARA O COMITÊ GESTOR DO IBS</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE FPE - PRINC. - FUNDEB</t>
         </is>
       </c>
       <c r="U1193" t="n">
-        <v>-96620253</v>
+        <v>-2099559983</v>
       </c>
       <c r="V1193" t="n">
         <v>2027</v>
@@ -82781,7 +82781,7 @@
       </c>
       <c r="X1193" t="inlineStr">
         <is>
-          <t>Inclui IBS - Previsão de novas receitas na LOA 2027 em relação à LDO 2027</t>
+          <t>Receita de Dedução Receita - Cota-Parte FPE - Princ. - FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82800,7 +82800,7 @@
         </is>
       </c>
       <c r="D1194" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G1194" t="n">
         <v>9</v>
@@ -82815,7 +82815,7 @@
         <v>1</v>
       </c>
       <c r="K1194" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="L1194" t="n">
         <v>0</v>
@@ -82830,15 +82830,15 @@
         <v>0</v>
       </c>
       <c r="P1194" t="n">
-        <v>9711500102000</v>
+        <v>9711530102000</v>
       </c>
       <c r="Q1194" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE FPE - PRINC. - FUNDEB</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1194" t="n">
-        <v>-2099559983</v>
+        <v>-330174995</v>
       </c>
       <c r="V1194" t="n">
         <v>2027</v>
@@ -82850,7 +82850,7 @@
       </c>
       <c r="X1194" t="inlineStr">
         <is>
-          <t>Receita de Dedução Receita - Cota-Parte FPE - Princ. - FUNDEB</t>
+          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - Municípios.</t>
         </is>
       </c>
     </row>
@@ -82869,7 +82869,7 @@
         </is>
       </c>
       <c r="D1195" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G1195" t="n">
         <v>9</v>
@@ -82893,21 +82893,21 @@
         <v>1</v>
       </c>
       <c r="N1195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1195" t="n">
         <v>0</v>
       </c>
       <c r="P1195" t="n">
-        <v>9711530102000</v>
+        <v>9711530103000</v>
       </c>
       <c r="Q1195" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - FUNDEB</t>
         </is>
       </c>
       <c r="U1195" t="n">
-        <v>-330174995</v>
+        <v>-198104997</v>
       </c>
       <c r="V1195" t="n">
         <v>2027</v>
@@ -82919,7 +82919,7 @@
       </c>
       <c r="X1195" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - Municípios.</t>
+          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - FUNDEB</t>
         </is>
       </c>
     </row>
@@ -82938,7 +82938,7 @@
         </is>
       </c>
       <c r="D1196" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G1196" t="n">
         <v>9</v>
@@ -82953,7 +82953,7 @@
         <v>1</v>
       </c>
       <c r="K1196" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L1196" t="n">
         <v>0</v>
@@ -82962,21 +82962,21 @@
         <v>1</v>
       </c>
       <c r="N1196" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O1196" t="n">
         <v>0</v>
       </c>
       <c r="P1196" t="n">
-        <v>9711530103000</v>
+        <v>9711540102000</v>
       </c>
       <c r="Q1196" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE IPI - ESTADOS EXPORT. PROD. INDUST. - PRINC. - FUNDEB</t>
+          <t>DEDUÇÃO REC. - COTA-PARTE CIDE - PRINC. - MUNICÍPIOS</t>
         </is>
       </c>
       <c r="U1196" t="n">
-        <v>-198104997</v>
+        <v>-29360522</v>
       </c>
       <c r="V1196" t="n">
         <v>2027</v>
@@ -82988,7 +82988,7 @@
       </c>
       <c r="X1196" t="inlineStr">
         <is>
-          <t>Receita de Dedução Rec. - Cota-Parte IPI - Estados Export. Prod. Indust. - Princ. - FUNDEB</t>
+          <t>Receita de Dedução Receita - Cota-Parte CIDE - Princ. - Municípios</t>
         </is>
       </c>
     </row>
@@ -83007,13 +83007,13 @@
         </is>
       </c>
       <c r="D1197" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="G1197" t="n">
         <v>9</v>
       </c>
       <c r="H1197" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I1197" t="n">
         <v>1</v>
@@ -83022,7 +83022,7 @@
         <v>1</v>
       </c>
       <c r="K1197" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="L1197" t="n">
         <v>0</v>
@@ -83031,21 +83031,21 @@
         <v>1</v>
       </c>
       <c r="N1197" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O1197" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P1197" t="n">
-        <v>9711540102000</v>
+        <v>9911010103004</v>
       </c>
       <c r="Q1197" t="inlineStr">
         <is>
-          <t>DEDUÇÃO REC. - COTA-PARTE CIDE - PRINC. - MUNICÍPIOS</t>
+          <t>DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
         </is>
       </c>
       <c r="U1197" t="n">
-        <v>-29360522</v>
+        <v>-11702813</v>
       </c>
       <c r="V1197" t="n">
         <v>2027</v>
@@ -83056,75 +83056,6 @@
         </is>
       </c>
       <c r="X1197" t="inlineStr">
-        <is>
-          <t>Receita de Dedução Receita - Cota-Parte CIDE - Princ. - Municípios</t>
-        </is>
-      </c>
-    </row>
-    <row r="1198">
-      <c r="A1198" t="n">
-        <v>9901</v>
-      </c>
-      <c r="B1198" t="inlineStr">
-        <is>
-          <t>RECEITA GERAL DO ESTADO</t>
-        </is>
-      </c>
-      <c r="C1198" t="inlineStr">
-        <is>
-          <t>RGE</t>
-        </is>
-      </c>
-      <c r="D1198" t="n">
-        <v>82</v>
-      </c>
-      <c r="G1198" t="n">
-        <v>9</v>
-      </c>
-      <c r="H1198" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1198" t="n">
-        <v>1</v>
-      </c>
-      <c r="J1198" t="n">
-        <v>1</v>
-      </c>
-      <c r="K1198" t="n">
-        <v>1</v>
-      </c>
-      <c r="L1198" t="n">
-        <v>0</v>
-      </c>
-      <c r="M1198" t="n">
-        <v>1</v>
-      </c>
-      <c r="N1198" t="n">
-        <v>3</v>
-      </c>
-      <c r="O1198" t="n">
-        <v>4</v>
-      </c>
-      <c r="P1198" t="n">
-        <v>9911010103004</v>
-      </c>
-      <c r="Q1198" t="inlineStr">
-        <is>
-          <t>DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
-        </is>
-      </c>
-      <c r="U1198" t="n">
-        <v>-11702813</v>
-      </c>
-      <c r="V1198" t="n">
-        <v>2027</v>
-      </c>
-      <c r="W1198" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X1198" t="inlineStr">
         <is>
           <t>RECeita de DEDUÇÃO REC. - MULTAS LEGISL. ESPECÍFICA - PRINC. - LEGISL. TRÂNSITO - COTA PARTE DO FUNDO NACIONAL DE SEGURANÇA E EDUCAÇÃO NO TRÂNSITO - FUNSET - ESTADO</t>
         </is>

</xml_diff>